<commit_message>
Round 3 follow-up: close more gaps (208 of 268 entries done)
- More independent holdout sources: links on other pages of the host,
  detail-page links, listing split before induction, missed-URL split
  before v2 widening; failed landings (404/5xx) are not positives
- Fixes: late <title> detection, v2 holdout pool, nav-region item lists,
  file-only landing pages, raw (undecoded) query values
- Complete traversal of 12 truncated sitemaps (prefix-filtered)
- YouGov economy/consumer reconciled: the listing UI hides the last batch;
  58 items fetched from the page's own read-only API and landed 200
- Forrester listing reconciled against the public REST total
- 142 verified rules covering 112 entries; 20 candidates; 45 entries
  remain blocked by the sites themselves

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HW9kjaADHDgTyps9HbQ9Ce
</commit_message>
<xml_diff>
--- a/url-pattern-verification/output/round3/result-table.xlsx
+++ b/url-pattern-verification/output/round3/result-table.xlsx
@@ -529,9 +529,9 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>S1-R2-E1 规则：R3-S1-R2-E1-F1 验证不通过（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）、标注测试有失败（留出 FN0/FP1））；链接 可打开（200，标题「Monthly Retail Trade - Main Page」）
+          <t>S1-R2-E1 规则：R3-S1-R2-E1-F1 验证不通过（机械门未通过：归纳正例 2&lt;3、标注测试有失败（留出 FN0/FP1）、留出指标 &lt;95%）；链接 可打开（200，标题「Monthly Retail Trade - Main Page」）
 S1-R2-E2 R3-S1-R2-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP1/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 12 个全部匹配
-S1-R2-E2 规则：R3-S1-R2-E2-F1 已验证；R3-S1-R2-E2-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「E-Commerce Statistics (E-STATS)」）</t>
+S1-R2-E2 规则：R3-S1-R2-E2-F1 已验证；R3-S1-R2-E2-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「E-Commerce Statistics (E-STATS)」）</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
@@ -649,7 +649,11 @@
 https://blogs.worldbank.org/en/home</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>^https://documents\.worldbank\.org/en/publication/documents\-reports/[a-z]+$</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>S1-R6-E1: https://www.worldbank.org/ext/en/development-topics
@@ -663,15 +667,19 @@
 S1-R6-E5: https://www.worldbank.org/ext/en/news
   其余 58 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R6-E5.txt
 S1-R6-E13: https://documents.worldbank.org/en/publication/documents-reports
-  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R6-E13.txt
+  其余 15 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R6-E13.txt
 S1-R6-E14: https://blogs.worldbank.org/en/home
   其余 49 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R6-E14.txt</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>S1-R6-E13 R3-S1-R6-E13-F1: https://documents.worldbank.org/en/publication/documents-reports/disclosure；https://documents.worldbank.org/en/publication/documents-reports/api（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留；E5 链接保留；E13 链接保留；E14 链接保留；E6 host免提；E7 host免提；E8 host免提；E9 host免提；E10 host免提；E11 host免提；E12 host免提</t>
+          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留；E5 链接保留；E13 正则+链接保留；E14 链接保留；E6 host免提；E7 host免提；E8 host免提；E9 host免提；E10 host免提；E11 host免提；E12 host免提</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -681,7 +689,8 @@
 S1-R6-E3 规则：无规则；链接 可打开（200，标题「Publications &amp; Research: Reports, Data, and More |」）
 S1-R6-E4 规则：无规则；链接 可打开（200，标题「What We Do | World Bank Group: Global Development,」）
 S1-R6-E5 规则：无规则；链接 可打开（200，标题「News | World Bank Group」）
-S1-R6-E13 规则：R3-S1-R6-E13-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Documents &amp; Reports - All Documents | The World Ba」）
+S1-R6-E13 R3-S1-R6-E13-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN5；覆盖检查：列表 4 个、sitemap 同结构 0 个全部匹配
+S1-R6-E13 规则：R3-S1-R6-E13-F1 已验证；链接 可打开（200，标题「Documents &amp; Reports - All Documents | The World Ba」）
 S1-R6-E14 规则：无规则；链接 可打开（200，标题「Unlock Development Insights with World Bank Blogs」）</t>
         </is>
       </c>
@@ -880,7 +889,7 @@
           <t>S1-R16-E1: https://www.bis.org/publications
   其余 2475 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R16-E1.txt
 S1-R16-E2: https://www.bis.org/statistics
-  其余 82 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R16-E2.txt
+  其余 84 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R16-E2.txt
 S1-R16-E4: https://www.bis.org/speeches
   其余 129 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R16-E4.txt
 S1-R16-E5: https://www.bis.org/committees/overview
@@ -934,7 +943,7 @@
         <is>
           <t>S1-R16-E1: 完整（列表+sitemap 合并枚举）：静态请求 510 页（入口+分页），未完成分页 0；前缀 /publications/ 下家族 2 个、成员 5074；前缀外同站链接 2475、文件 0；sitemap 中同结构但不在列表的 URL：F1=14、F2=2
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R16-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /statistics/ 下家族 0 个、成员 0；前缀外同站链接 35、文件 46；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+S1-R16-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /statistics/ 下家族 0 个、成员 0；前缀外同站链接 35、文件 46；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R16-E4: 完整（列表+sitemap 合并枚举）：静态请求 77 页（入口+分页），未完成分页 0；前缀 /speeches/ 下家族 1 个、成员 760；前缀外同站链接 127、文件 0；sitemap 中同结构但不在列表的 URL：F1=21674
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -985,8 +994,12 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.itu\.int/en/ITU\-R/[a-z-]+/[a-zA-Z0-9-]+/Pages/[a-zA-Z0-9-]+\.aspx$
-^https://www\.itu\.int/en/ITU\-T/[a-zA-Z-]+/Pages/[a-z]+\.aspx$</t>
+          <t>^https://www\.itu\.int/itu\-d/sites/statistics/[a-z-]+/$
+^https://www\.itu\.int/en/ITU\-R/seminars/rrs/[a-zA-Z0-9%-]+/Pages/default\.aspx$
+^https://www\.itu\.int/en/ITU\-R/[a-z-]+/[a-zA-Z0-9-]+/Pages/[a-zA-Z0-9-]+\.aspx$
+^https://www\.itu\.int/en/ITU\-T/[a-zA-Z-]+/Pages/[a-z]+\.aspx$
+^https://www\.itu\.int/en/ITU\-T/[a-z0-9]+/[a-z0-9-]+/Pages/default\.aspx$
+^https://www\.itu\.int/hub/news/[a-z-]+/$</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -998,39 +1011,47 @@
 S1-R18-E4: https://www.itu.int/en/action/Pages/default.aspx
   其余 61 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E4.txt
 S1-R18-E5: https://www.itu.int/en/ITU-R/Pages/default.aspx
-  其余 142 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E5.txt
+  其余 136 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E5.txt
 S1-R18-E6: https://www.itu.int/en/ITU-T/Pages/default.aspx
-  其余 49 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E6.txt
+  其余 46 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E6.txt
 S1-R18-E7: https://www.itu.int/en/ITU-D/Pages/default.aspx
   其余 82 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E7.txt
 S1-R18-E8: https://www.itu.int/hub/news/
-  其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E8.txt
+  其余 9 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E8.txt
 S1-R18-E9: https://www.itu.int/en/publications/Pages/media.aspx
   其余 52 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R18-E9.txt</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>S1-R18-E5 R3-S1-R18-E5-F4: https://www.itu.int/en/ITU-R/information/events/Pages/Fellowships.aspx；https://www.itu.int/en/ITU-R/seminars/ML-in-radio-prop/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）
-S1-R18-E6 R3-S1-R18-E6-F1: https://www.itu.int/en/ITU-T/AI/Pages/ai-repository.aspx；https://www.itu.int/en/ITU-T/NoW/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R18-E2 R3-S1-R18-E2-F1: https://www.itu.int/itu-d/sites/statistics/fr/；https://www.itu.int/itu-d/sites/statistics/ar/（已落地核验 200，公开访问，2026-10-26）
+S1-R18-E5 R3-S1-R18-E5-F2: https://www.itu.int/en/ITU-R/seminars/rrs/RRS-26-Americas/Pages/default.aspx；https://www.itu.int/en/ITU-R/seminars/rrs/RRS-26-Europe/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）
+S1-R18-E5 R3-S1-R18-E5-F4: https://www.itu.int/en/ITU-R/information/events/Pages/Fellowships.aspx；https://www.itu.int/en/ITU-R/seminars/ML-in-radio-prop/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）
+S1-R18-E6 R3-S1-R18-E6-F1: https://www.itu.int/en/ITU-T/AI/Pages/ai-repository.aspx；https://www.itu.int/en/ITU-T/NoW/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）
+S1-R18-E6 R3-S1-R18-E6-F2: https://www.itu.int/en/ITU-T/focusgroups/ai4a/Pages/default.aspx；https://www.itu.int/en/ITU-T/extcoop/ai4resilience/Pages/default.aspx（已落地核验 200，公开访问，2026-10-26）
+S1-R18-E8 R3-S1-R18-E8-F1: https://www.itu.int/hub/news/impact-videos/；https://www.itu.int/hub/news/did-you-know/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E4 链接保留；E5 正则+链接保留；E6 正则+链接保留；E7 链接保留；E8 链接保留；E9 链接保留；E3 host免提</t>
+          <t>E1 链接保留；E2 正则+链接保留；E4 链接保留；E5 正则+链接保留；E6 正则+链接保留；E7 链接保留；E8 正则+链接保留；E9 链接保留；E3 host免提</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
           <t>S1-R18-E1 规则：无规则；链接 可打开（200，标题「ITU Publications / UN agency for digital technolog」）
-S1-R18-E2 规则：无规则；链接 可打开（200，标题「ITU-D ICT Statistics」）
+S1-R18-E2 R3-S1-R18-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN4；覆盖检查：列表 5 个、sitemap 同结构 0 个全部匹配
+S1-R18-E2 规则：R3-S1-R18-E2-F1 已验证；链接 可打开（200，标题「ITU-D ICT Statistics」）
 S1-R18-E4 规则：R3-S1-R18-E4-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Key Areas of Action」）
+S1-R18-E5 R3-S1-R18-E5-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN6；覆盖检查：列表 6 个、sitemap 同结构 0 个全部匹配
 S1-R18-E5 R3-S1-R18-E5-F4 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN6；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
-S1-R18-E5 规则：R3-S1-R18-E5-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R18-E5-F4 已验证；链接 可打开（200，标题「ITU Radiocommunication Sector」）
+S1-R18-E5 规则：R3-S1-R18-E5-F2 已验证；R3-S1-R18-E5-F4 已验证；链接 可打开（200，标题「ITU Radiocommunication Sector」）
 S1-R18-E6 R3-S1-R18-E6-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP4/FP0/FN0/TN6；覆盖检查：列表 25 个、sitemap 同结构 0 个全部匹配
-S1-R18-E6 规则：R3-S1-R18-E6-F1 已验证；R3-S1-R18-E6-F2 部分验证（候选）（机械门未通过：留出反例 2&lt;3）；链接 可打开（200，标题「ITU Telecommunication Standardization Sector」）
+S1-R18-E6 R3-S1-R18-E6-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP1/FP0/FN0/TN6；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
+S1-R18-E6 规则：R3-S1-R18-E6-F1 已验证；R3-S1-R18-E6-F2 已验证；链接 可打开（200，标题「ITU Telecommunication Standardization Sector」）
 S1-R18-E7 规则：R3-S1-R18-E7-F1 验证不通过（机械门未通过：标注测试有失败（留出 FN0/FP1）、留出指标 &lt;95%）；链接 可打开（200，标题「ITU Telecommunication Development Sector」）
-S1-R18-E8 规则：R3-S1-R18-E8-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「ITU News: Latest from the UN agency for digital te」）
+S1-R18-E8 R3-S1-R18-E8-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN4；覆盖检查：列表 4 个、sitemap 同结构 0 个全部匹配
+S1-R18-E8 规则：R3-S1-R18-E8-F1 已验证；链接 可打开（200，标题「ITU News: Latest from the UN agency for digital te」）
 S1-R18-E9 规则：无规则；链接 可打开（200，标题「Catalogue of Publications」）</t>
         </is>
       </c>
@@ -1050,7 +1071,7 @@
         <is>
           <t>S1-R18-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 82；前缀 /hub/pubs/ 下家族 0 个、成员 0；前缀外同站链接 20、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R18-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 100；前缀 /itu-d/sites/statistics/ 下家族 0 个、成员 0；前缀外同站链接 14、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+S1-R18-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 100；前缀 /itu-d/sites/statistics/ 下家族 1 个、成员 5；前缀外同站链接 14、文件 0；sitemap 中同结构但不在列表的 URL：F1=0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R18-E4: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/action/ 下家族 2 个、成员 11；前缀外同站链接 50、文件 0；sitemap 中同结构但不在列表的 URL：F2=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -1114,10 +1135,19 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.wipo\.int/en/web/economics/[a-z-]+$
+          <t>^https://www\.wipo\.int/en/web/global\-brand\-database/w/news/[0-9]+/[a-z0-9_-]+$
+^https://www\.wipo\.int/en/web/patent\-analytics/w/[a-z]+/2026/[a-z0-9-]+$
+^https://www\.wipo\.int/en/web/business/w/news/2026/[a-z0-9-]+$
+^https://www\.wipo\.int/en/web/economics/[a-z-]+$
 ^https://www\.wipo\.int/en/web/technology\-transfer/[a-z-]+$
 ^https://www\.wipo\.int/en/web/technology\-transfer/w/stories/[a-z0-9-]+$
-^https://www\.wipo\.int/en/web/global\-innovation\-index/[0-9]+/[a-z-]+$</t>
+^https://www\.wipo\.int/en/web/wipo\-magazine/articles/[a-z0-9-]+$
+^https://www\.wipo\.int/en/web/ip\-advantage/w/stories/[a-z0-9-]+$
+^https://www\.wipo\.int/en/web/ip\-advantage/[a-z-]+$
+^https://www\.wipo\.int/en/web/global\-innovation\-index/w/[a-z]+/2026/[a-z0-9-]+$
+^https://www\.wipo\.int/en/web/global\-innovation\-index/[0-9]+/[a-z-]+$
+^https://www\.wipo\.int/en/web/world\-ip\-report/[0-9]+/index$
+^https://www3\.wipo\.int/ipstats/key\-search/search\-result\?type=KEY&amp;key=[0-9]*$</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -1131,15 +1161,15 @@
 S1-R19-E4: https://www.wipo.int/en/web/patentscope/
   其余 166 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E4.txt
 S1-R19-E6: https://www.wipo.int/en/web/global-brand-database
-  其余 157 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E6.txt
+  其余 154 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E6.txt
 S1-R19-E8: https://www.wipo.int/en/web/global-design-database
   其余 153 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E8.txt
 S1-R19-E10: https://www.wipo.int/en/web/patent-analytics
-  其余 180 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E10.txt
+  其余 173 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E10.txt
 S1-R19-E11: https://www.wipo.int/en/web/wipolex
   其余 158 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E11.txt
 S1-R19-E12: https://www.wipo.int/en/web/business
-  其余 165 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E12.txt
+  其余 158 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E12.txt
 S1-R19-E13: https://www.wipo.int/en/web/economics
   其余 142 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E13.txt
 S1-R19-E14: https://www.wipo.int/en/web/technology-transfer
@@ -1157,69 +1187,87 @@
 S1-R19-E20: https://www.wipo.int/en/web/frontier-technologies
   其余 141 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E20.txt
 S1-R19-E21: https://www.wipo.int/en/web/wipo-magazine
-  其余 148 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E21.txt
+  其余 134 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E21.txt
 S1-R19-E22: https://www.wipo.int/en/web/ip-advantage
-  其余 163 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E22.txt
+  其余 130 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E22.txt
 S1-R19-E23: https://www.wipo.int/en/web/technology-trends
   其余 138 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E23.txt
 S1-R19-E24: https://www.wipo.int/en/web/global-innovation-index
-  其余 160 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E24.txt
+  其余 153 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E24.txt
 S1-R19-E25: https://www.wipo.int/en/web/world-ip-report
-  其余 147 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E25.txt
+  其余 143 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E25.txt
 S1-R19-E26: https://www.wipo.int/en/web/country-profiles
   其余 133 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E26.txt
 S1-R19-E27: https://www3.wipo.int/madrid/monitor/en/
   其余 25 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E27.txt
 S1-R19-E28: https://www3.wipo.int/ipstats/
-  其余 16 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E28.txt
+  其余 5 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E28.txt
 S1-R19-E29: https://www.wipo.int/en/web/patentscope/data/index
   其余 150 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R19-E29.txt</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>S1-R19-E13 R3-S1-R19-E13-F1: https://www.wipo.int/en/web/economics/music-insights；https://www.wipo.int/en/web/economics/creative-industries-insights（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R19-E6 R3-S1-R19-E6-F2: https://www.wipo.int/en/web/global-brand-database/w/news/2024/trademarks-of-saint-vincent-and-the-grenadines-now-available-in-the-global-brand-database；https://www.wipo.int/en/web/global-brand-database/w/news/2025/trademarks-of-croatia-are-now-available-in-the-global-brand-database（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E10 R3-S1-R19-E10-F1: https://www.wipo.int/en/web/patent-analytics/w/news/2026/wipo-launches-new-e-tutorial-on-patent-analytics；https://www.wipo.int/en/web/patent-analytics/w/blog/2026/beyond-the-chatbot-what-patent-data-reveals-about-the-next-phase-of-genai（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E12 R3-S1-R19-E12-F2: https://www.wipo.int/en/web/business/w/news/2026/wipo-and-myipo-establish-joint-ip-business-center；https://www.wipo.int/en/web/business/w/news/2026/ipmc-shanghai-yangtze-river-delta-green-technology-intellectual-property-management-clinic-ipmc-officially-launches（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E13 R3-S1-R19-E13-F1: https://www.wipo.int/en/web/economics/music-insights；https://www.wipo.int/en/web/economics/creative-industries-insights（已落地核验 200，公开访问，2026-10-26）
 S1-R19-E14 R3-S1-R19-E14-F1: https://www.wipo.int/en/web/technology-transfer/ipr-management-principles；https://www.wipo.int/en/web/technology-transfer/academic-assets-management（已落地核验 200，公开访问，2026-10-26）
 S1-R19-E14 R3-S1-R19-E14-F3: https://www.wipo.int/en/web/technology-transfer/w/stories/ip-policy-hashemite-university；https://www.wipo.int/en/web/technology-transfer/w/stories/sadc-technology-transfer-mentorship-program-building-regional-capacity（已落地核验 200，公开访问，2026-10-26）
-S1-R19-E24 R3-S1-R19-E24-F2: https://www.wipo.int/en/web/global-innovation-index/2021/index；https://www.wipo.int/en/web/global-innovation-index/2024/index（已落地核验 200，公开访问，2026-10-26）</t>
+S1-R19-E21 R3-S1-R19-E21-F1: https://www.wipo.int/en/web/wipo-magazine/articles/how-saudi-producer-ahmed-alsallal-uses-music-to-promote-intellectual-property-74728；https://www.wipo.int/en/web/wipo-magazine/articles/combatting-ai-deepfakes-to-safeguard-indian-cricketers-image-rights-100827（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E22 R3-S1-R19-E22-F1: https://www.wipo.int/en/web/ip-advantage/w/stories/elevating-bandung-sweet-legacy-through-innovation-and-ip；https://www.wipo.int/en/web/ip-advantage/w/stories/fourier-healthcare-robots-with-humanoid-designs（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E22 R3-S1-R19-E22-F2: https://www.wipo.int/en/web/ip-advantage/pct-system-stories；https://www.wipo.int/en/web/ip-advantage/asia-pacific-region-stories（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E24 R3-S1-R19-E24-F1: https://www.wipo.int/en/web/global-innovation-index/w/blogs/2026/lights-camera-records-global-film-production；https://www.wipo.int/en/web/global-innovation-index/w/blogs/2026/international-trade-in-ideas-know-how-and-intellectual-property（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E24 R3-S1-R19-E24-F2: https://www.wipo.int/en/web/global-innovation-index/2021/index；https://www.wipo.int/en/web/global-innovation-index/2024/index（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E25 R3-S1-R19-E25-F1: https://www.wipo.int/en/web/world-ip-report/2019/index；https://www.wipo.int/en/web/world-ip-report/2022/index（已落地核验 200，公开访问，2026-10-26）
+S1-R19-E28 R3-S1-R19-E28-F1: https://www3.wipo.int/ipstats/key-search/search-result?type=KEY&amp;key=201；https://www3.wipo.int/ipstats/key-search/search-result?type=KEY&amp;key=222（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留；E6 链接保留；E8 链接保留；E10 链接保留；E11 链接保留；E12 链接保留；E13 正则+链接保留；E14 正则+链接保留；E15 链接保留；E16 链接保留；E17 链接保留；E18 链接保留；E19 链接保留；E20 链接保留；E21 链接保留；E22 链接保留；E23 链接保留；E24 正则+链接保留；E25 链接保留；E26 链接保留；E27 链接保留；E28 链接保留；E29 链接保留；E5 host免提；E7 host免提；E9 host免提</t>
+          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留；E6 正则+链接保留；E8 链接保留；E10 正则+链接保留；E11 链接保留；E12 正则+链接保留；E13 正则+链接保留；E14 正则+链接保留；E15 链接保留；E16 链接保留；E17 链接保留；E18 链接保留；E19 链接保留；E20 链接保留；E21 正则+链接保留；E22 正则+链接保留；E23 链接保留；E24 正则+链接保留；E25 正则+链接保留；E26 链接保留；E27 链接保留；E28 正则+链接保留；E29 链接保留；E5 host免提；E7 host免提；E9 host免提</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
           <t>S1-R19-E1 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP Resources」）
 S1-R19-E2 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Publications」）
-S1-R19-E3 规则：R3-S1-R19-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Statistics」）
-S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）；归纳样本跳到其他页面 1）；R3-S1-R19-E4-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
-S1-R19-E6 规则：R3-S1-R19-E6-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E6-F2 部分验证（候选）（机械门未通过：留出反例 1&lt;3）；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Brand Database」）
-S1-R19-E8 规则：R3-S1-R19-E8-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Design Database」）
-S1-R19-E10 规则：R3-S1-R19-E10-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E10-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Patent Analytics」）
+S1-R19-E3 规则：R3-S1-R19-E3-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Statistics」）
+S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）；归纳样本跳到家族外页面 1：https://www.wipo.int/en/web/patentscope/webinar → https://www.wipo.int/en/web/patentscope/webinar/index）；R3-S1-R19-E4-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
+S1-R19-E6 R3-S1-R19-E6-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP3/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
+S1-R19-E6 规则：R3-S1-R19-E6-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E6-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Brand Database」）
+S1-R19-E8 规则：R3-S1-R19-E8-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Design Database」）
+S1-R19-E10 R3-S1-R19-E10-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN6；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
+S1-R19-E10 规则：R3-S1-R19-E10-F1 已验证；R3-S1-R19-E10-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Patent Analytics」）
 S1-R19-E11 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Lex – A Global IP Law Database」）
-S1-R19-E12 规则：R3-S1-R19-E12-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）；列表成员漏配 1）；R3-S1-R19-E12-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Why Intellectual Property is Essential for your Bu」）
+S1-R19-E12 R3-S1-R19-E12-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN6；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
+S1-R19-E12 规则：R3-S1-R19-E12-F1 部分验证（候选）（机械门未通过：留出与归纳/回归重叠；列表成员漏配 1）；R3-S1-R19-E12-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Why Intellectual Property is Essential for your Bu」）
 S1-R19-E13 R3-S1-R19-E13-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP1/FP0/FN0/TN7；覆盖检查：列表 11 个、sitemap 同结构 0 个全部匹配
 S1-R19-E13 规则：R3-S1-R19-E13-F1 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP and Economics」）
 S1-R19-E14 R3-S1-R19-E14-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP2/FP0/FN0/TN7；覆盖检查：列表 10 个、sitemap 同结构 0 个全部匹配
 S1-R19-E14 R3-S1-R19-E14-F3 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP2/FP0/FN0/TN6；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
-S1-R19-E14 规则：R3-S1-R19-E14-F1 已验证；R3-S1-R19-E14-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E14-F3 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Knowledge and Technology Transfer」）
+S1-R19-E14 规则：R3-S1-R19-E14-F1 已验证；R3-S1-R19-E14-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E14-F3 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Knowledge and Technology Transfer」）
 S1-R19-E15 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP Commercialization: Taking Research from Lab to 」）
-S1-R19-E16 规则：R3-S1-R19-E16-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E16-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Finance」）
+S1-R19-E16 规则：R3-S1-R19-E16-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E16-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Finance」）
 S1-R19-E17 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intangible Assets and IP」）
 S1-R19-E18 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP in the Innovation Ecosystem」）
 S1-R19-E19 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property and Competition Policy」）
-S1-R19-E20 规则：R3-S1-R19-E20-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP and Frontier Technologies」）
-S1-R19-E21 规则：R3-S1-R19-E21-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Magazine」）
-S1-R19-E22 规则：R3-S1-R19-E22-F1 部分验证（候选）（机械门未通过：留出反例 2&lt;3）；R3-S1-R19-E22-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Case Studies on Intellectual Property (IP Advantag」）
+S1-R19-E20 规则：R3-S1-R19-E20-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP and Frontier Technologies」）
+S1-R19-E21 R3-S1-R19-E21-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP3/FP0/FN0/TN4；覆盖检查：列表 14 个、sitemap 同结构 0 个全部匹配
+S1-R19-E21 规则：R3-S1-R19-E21-F1 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Magazine」）
+S1-R19-E22 R3-S1-R19-E22-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN6；覆盖检查：列表 26 个、sitemap 同结构 0 个全部匹配
+S1-R19-E22 R3-S1-R19-E22-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
+S1-R19-E22 规则：R3-S1-R19-E22-F1 已验证；R3-S1-R19-E22-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Case Studies on Intellectual Property (IP Advantag」）
 S1-R19-E23 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Technology Trends」）
+S1-R19-E24 R3-S1-R19-E24-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN6；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
 S1-R19-E24 R3-S1-R19-E24-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP4/FP0/FN0/TN6；覆盖检查：列表 5 个、sitemap 同结构 0 个全部匹配
-S1-R19-E24 规则：R3-S1-R19-E24-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E24-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Innovation Index」）
-S1-R19-E25 规则：R3-S1-R19-E25-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「World Intellectual Property Report」）
+S1-R19-E24 规则：R3-S1-R19-E24-F1 已验证；R3-S1-R19-E24-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Innovation Index」）
+S1-R19-E25 R3-S1-R19-E25-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN4；覆盖检查：列表 4 个、sitemap 同结构 0 个全部匹配
+S1-R19-E25 规则：R3-S1-R19-E25-F1 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「World Intellectual Property Report」）
 S1-R19-E26 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Country IP Profiles」）
 S1-R19-E27 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Madrid Monitor」）
-S1-R19-E28 规则：R3-S1-R19-E28-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）、留出反例 2&lt;3）；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO IP Statistics Data Center」）
+S1-R19-E28 R3-S1-R19-E28-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP2/FP0/FN0/TN5；覆盖检查：列表 11 个、sitemap 同结构 0 个全部匹配
+S1-R19-E28 规则：R3-S1-R19-E28-F1 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO IP Statistics Data Center」）
 S1-R19-E29 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PCT Data Products and Services」）</t>
         </is>
       </c>
@@ -1355,24 +1403,30 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.epo\.org/en/searching\-for\-patents/helpful\-resources/patent\-knowledge\-news/[a-z0-9-]+$
-^https://www\.epo\.org/en/news\-events/[a-z-]+/[a-z0-9-]+$</t>
+          <t>^https://www\.epo\.org/en/searching\-for\-patents/[a-z-]+/[a-z-]+$
+^https://www\.epo\.org/en/searching\-for\-patents/[a-z-]+$
+^https://www\.epo\.org/en/searching\-for\-patents/helpful\-resources/patent\-knowledge\-news/[a-z0-9-]+$
+^https://www\.epo\.org/en/news\-events/[a-z-]+/[a-z0-9-]+$
+^https://www\.epo\.org/en/news\-events/[a-z-]+$</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>S1-R20-E1: https://www.epo.org/en/searching-for-patents
-  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R20-E1.txt
+  其余 4 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R20-E1.txt
 S1-R20-E2: https://www.epo.org/en/news-events
-  其余 12 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R20-E2.txt
+  其余 5 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R20-E2.txt
 S1-R20-E3: https://www.epo.org/en/results?filters=%5B%5D&amp;sortField=&amp;sortDirection=&amp;tab=all_results
   其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R20-E3.txt</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>S1-R20-E1 R3-S1-R20-E1-F3: https://www.epo.org/en/searching-for-patents/helpful-resources/patent-knowledge-news/accelerated-examination-and-speedy；https://www.epo.org/en/searching-for-patents/helpful-resources/patent-knowledge-news/changes-vietnamese-patent-law（已落地核验 200，公开访问，2026-10-26）
-S1-R20-E2 R3-S1-R20-E2-F1: https://www.epo.org/en/news-events/events/upcoming-myepo-services-seminars；https://www.epo.org/en/news-events/events/boards-appeal-case-law-conference-2026（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R20-E1 R3-S1-R20-E1-F1: https://www.epo.org/en/searching-for-patents/business/technology-insight-reports；https://www.epo.org/en/searching-for-patents/helpful-resources/business-and-statistics（已落地核验 200，公开访问，2026-10-26）
+S1-R20-E1 R3-S1-R20-E1-F2: https://www.epo.org/en/searching-for-patents/data；https://www.epo.org/en/searching-for-patents/business（已落地核验 200，公开访问，2026-10-26）
+S1-R20-E1 R3-S1-R20-E1-F3: https://www.epo.org/en/searching-for-patents/helpful-resources/patent-knowledge-news/accelerated-examination-and-speedy；https://www.epo.org/en/searching-for-patents/helpful-resources/patent-knowledge-news/changes-vietnamese-patent-law（已落地核验 200，公开访问，2026-10-26）
+S1-R20-E2 R3-S1-R20-E2-F1: https://www.epo.org/en/news-events/events/upcoming-myepo-services-seminars；https://www.epo.org/en/news-events/events/boards-appeal-case-law-conference-2026（已落地核验 200，公开访问，2026-10-26）
+S1-R20-E2 R3-S1-R20-E2-F2: https://www.epo.org/en/news-events/european-inventor-award；https://www.epo.org/en/news-events/events（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1382,10 +1436,13 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>S1-R20-E1 R3-S1-R20-E1-F3 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 3 个、sitemap 同结构 258 个全部匹配
-S1-R20-E1 规则：R3-S1-R20-E1-F1 部分验证（候选）（机械门未通过：有正例未完成落地身份核验）；R3-S1-R20-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R20-E1-F3 已验证；链接 可打开（200，标题「Searching for patents | epo.org」）
+          <t>S1-R20-E1 R3-S1-R20-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 9 个、sitemap 同结构 28 个全部匹配
+S1-R20-E1 R3-S1-R20-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 6 个、sitemap 同结构 6 个全部匹配
+S1-R20-E1 R3-S1-R20-E1-F3 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 3 个、sitemap 同结构 258 个全部匹配
+S1-R20-E1 规则：R3-S1-R20-E1-F1 已验证；R3-S1-R20-E1-F2 已验证；R3-S1-R20-E1-F3 已验证；链接 可打开（200，标题「Searching for patents | epo.org」）
 S1-R20-E2 R3-S1-R20-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 9 个、sitemap 同结构 1087 个全部匹配
-S1-R20-E2 规则：R3-S1-R20-E2-F1 已验证；R3-S1-R20-E2-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「News &amp; events | epo.org」）
+S1-R20-E2 R3-S1-R20-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 7 个、sitemap 同结构 7 个全部匹配
+S1-R20-E2 规则：R3-S1-R20-E2-F1 已验证；R3-S1-R20-E2-F2 已验证；链接 可打开（200，标题「News &amp; events | epo.org」）
 S1-R20-E3 规则：无规则；链接 可打开（200，标题「| epo.org」）</t>
         </is>
       </c>
@@ -1398,9 +1455,9 @@
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>S1-R20-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/searching-for-patents/ 下家族 3 个、成员 18；前缀外同站链接 4、文件 0；sitemap 中同结构但不在列表的 URL：F1=19、F2=0、F3=255
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R20-E2: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/news-events/ 下家族 2 个、成员 16；前缀外同站链接 5、文件 0；sitemap 中同结构但不在列表的 URL：F1=1078、F2=0
+          <t>S1-R20-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/searching-for-patents/ 下家族 3 个、成员 18；前缀外同站链接 4、文件 0；sitemap 中同结构但不在列表的 URL：F1=19、F2=0、F3=255
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R20-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/news-events/ 下家族 2 个、成员 16；前缀外同站链接 5、文件 0；sitemap 中同结构但不在列表的 URL：F1=1078、F2=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R20-E3: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 1080；前缀 /en/results/ 下家族 0 个、成员 0；前缀外同站链接 2、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -1617,7 +1674,8 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.euromonitor\.com/insights/[a-z-]+$</t>
+          <t>^https://www\.euromonitor\.com/insights/[a-z-]+$
+^https://www\.euromonitor\.com/store/explore\-reports/[a-z-]+/[a-z-]+$</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -1627,25 +1685,27 @@
 S1-R27-E2: https://www.euromonitor.com/webinar
   其余 117 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R27-E2.txt
 S1-R27-E3: https://www.euromonitor.com/store/explore-reports
-  其余 46 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R27-E3.txt</t>
+  其余 30 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R27-E3.txt</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>S1-R27-E1 R3-S1-R27-E1-F1: https://www.euromonitor.com/insights/digital；https://www.euromonitor.com/insights/consumer-foodservice（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R27-E1 R3-S1-R27-E1-F1: https://www.euromonitor.com/insights/digital；https://www.euromonitor.com/insights/consumer-foodservice（已落地核验 200，公开访问，2026-10-26）
+S1-R27-E3 R3-S1-R27-E3-F1: https://www.euromonitor.com/store/explore-reports/asia-pacific/uzbekistan；https://www.euromonitor.com/store/explore-reports/consumer-health/digestive-remedies（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 链接保留；E3 链接保留</t>
+          <t>E1 正则+链接保留；E2 链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
           <t>S1-R27-E1 R3-S1-R27-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP5/FP0/FN0/TN7；覆盖检查：列表 28 个、sitemap 同结构 33 个全部匹配
-S1-R27-E1 规则：R3-S1-R27-E1-F1 已验证；R3-S1-R27-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Insights is Our Market Research and Business Intel」）
+S1-R27-E1 规则：R3-S1-R27-E1-F1 已验证；R3-S1-R27-E1-F2 部分验证（候选）（机械门未通过：留出与归纳/回归重叠）；链接 可打开（200，标题「Insights is Our Market Research and Business Intel」）
 S1-R27-E2 规则：无规则；链接 可打开（200，标题「Market Research, Data Analysis and Business Intell」）
-S1-R27-E3 规则：R3-S1-R27-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Explore reports - Euromonitor.com」）</t>
+S1-R27-E3 R3-S1-R27-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP4/FP0/FN0/TN6；覆盖检查：列表 16 个、sitemap 同结构 0 个全部匹配
+S1-R27-E3 规则：R3-S1-R27-E3-F1 已验证；链接 可打开（200，标题「Explore reports - Euromonitor.com」）</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1734,25 +1794,37 @@
 https://www.nielsen.com/news-center/</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.nielsen\.com/insights/[a-z0-9]+/[a-z0-9%_-]+/$
+^https://www\.nielsen\.com/news\-center/2026/[a-z0-9-]+/$</t>
+        </is>
+      </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
           <t>S1-R30-E1: https://www.nielsen.com/insights/
-  其余 16 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R30-E1.txt
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R30-E1.txt
 S1-R30-E2: https://www.nielsen.com/news-center/
-  其余 9 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R30-E2.txt</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="inlineStr"/>
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R30-E2.txt</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>S1-R30-E1 R3-S1-R30-E1-F1: https://www.nielsen.com/insights/2010/age-matters-mobile-youth-in-vietnam/；https://www.nielsen.com/insights/2025/what-are-nielsen-ratings/（已落地核验 200，公开访问，2026-10-26）
+S1-R30-E2 R3-S1-R30-E2-F1: https://www.nielsen.com/news-center/2026/football-and-younger-viewers-drive-ad-supported-tv-viewing-to-2025-high-nielsens-q4-2025-ad-supported-gauge-finds/；https://www.nielsen.com/news-center/2026/mcdonalds-takes-top-spot-as-new-zealands-fast-food-tastes-evolve-according-to-nielsen/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>S1-R30-E1 规则：R3-S1-R30-E1-F1 部分验证（候选）（机械门未通过：有正例未完成落地身份核验）；链接 可打开（200，标题「Insights | Nielsen」）
-S1-R30-E2 规则：R3-S1-R30-E2-F1 部分验证（候选）（机械门未通过：有正例未完成落地身份核验）；链接 可打开（200，标题「News Center Archive | Nielsen」）</t>
+          <t>S1-R30-E1 R3-S1-R30-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 16 个、sitemap 同结构 3027 个全部匹配
+S1-R30-E1 规则：R3-S1-R30-E1-F1 已验证；链接 可打开（200，标题「Insights | Nielsen」）
+S1-R30-E2 R3-S1-R30-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 9 个、sitemap 同结构 109 个全部匹配
+S1-R30-E2 规则：R3-S1-R30-E2-F1 已验证；链接 可打开（200，标题「News Center Archive | Nielsen」）</t>
         </is>
       </c>
       <c r="G30" s="3" t="inlineStr">
@@ -1763,9 +1835,9 @@
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>S1-R30-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /insights/ 下家族 1 个、成员 16；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=3015
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R30-E2: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /news-center/ 下家族 1 个、成员 9；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=100
+          <t>S1-R30-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /insights/ 下家族 1 个、成员 16；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=3015
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R30-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /news-center/ 下家族 1 个、成员 9；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=100
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -1932,27 +2004,36 @@
 https://www.circana.com/news</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.circana\.com/industries/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>S1-R34-E1: https://www.circana.com/insights
   其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R34-E1.txt
 S1-R34-E2: https://www.circana.com/industries
-  其余 33 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R34-E2.txt
+  其余 3 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R34-E2.txt
 S1-R34-E3: https://www.circana.com/news
-  其余 34 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R34-E3.txt</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr"/>
+  其余 37 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R34-E3.txt</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>S1-R34-E2 R3-S1-R34-E2-F1: https://www.circana.com/industries/alcoholic-beverages；https://www.circana.com/industries/center-store-and-frozen-foods（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 链接保留</t>
+          <t>E1 链接保留；E2 正则+链接保留；E3 链接保留</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
           <t>S1-R34-E1 规则：无规则；链接 可打开（200，标题「Home | Insights」）
-S1-R34-E2 规则：无规则；链接 可打开（200，标题「Industries Circana Provides Market, Survey &amp; Consu」）
+S1-R34-E2 R3-S1-R34-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN5；覆盖检查：列表 30 个、sitemap 同结构 30 个全部匹配
+S1-R34-E2 规则：R3-S1-R34-E2-F1 已验证；链接 可打开（200，标题「Industries Circana Provides Market, Survey &amp; Consu」）
 S1-R34-E3 规则：无规则；链接 可打开（200，标题「Circana Insights - get the latest news, insights, 」）</t>
         </is>
       </c>
@@ -1965,18 +2046,18 @@
       </c>
       <c r="H34" s="3" t="inlineStr">
         <is>
-          <t>S1-R34-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 8；前缀 /insights/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R34-E2: 完整：静态请求 1 页（入口+分页），未完成分页 0；前缀 /industries/ 下家族 1 个、成员 30；前缀外同站链接 3、文件 0
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R34-E3: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 3 轮、点击加载更多 0 次、渲染后链接 448；前缀 /news/ 下家族 0 个、成员 0；前缀外同站链接 34、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+          <t>S1-R34-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 8；前缀 /insights/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；页面上没有可枚举的标准链接（a[href]），内容可能由脚本组件渲染
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R34-E2: 完整：静态请求 1 页（入口+分页），未完成分页 0；前缀 /industries/ 下家族 1 个、成员 30；前缀外同站链接 3、文件 0；sitemap 中同结构但不在列表的 URL：F1=0
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R34-E3: 完整：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 3 轮、点击加载更多 0 次、渲染后链接 448；前缀 /news/ 下家族 1 个、成员 3；前缀外同站链接 34、文件 0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
       <c r="I34" s="3" t="inlineStr">
         <is>
           <t>行边界为重建：内联粘贴丢失引号，按连续同注册域分组得 152 行（107 个 URL 单元格+45 个“/”行），与前轮检查点计数一致，待与原始文件核对
-S1-R34-E2 R3-S1-R34-E2-F1 未成规则：归纳样本落地不足 3 个正常页面</t>
+S1-R34-E3 R3-S1-R34-E3-F1 未成规则：归纳样本落地不足 3 个正常页面</t>
         </is>
       </c>
     </row>
@@ -1987,25 +2068,34 @@
 https://www.comscore.com/Insights/Presentations-and-Whitepapers</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr"/>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.comscore\.com/Insights/Presentations\-and\-Whitepapers/2026/[a-zA-Z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
           <t>S1-R35-E1: https://www.comscore.com/Insights/Blog
   其余 20 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R35-E1.txt
 S1-R35-E2: https://www.comscore.com/Insights/Presentations-and-Whitepapers
-  其余 20 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R35-E2.txt</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr"/>
+  其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R35-E2.txt</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>S1-R35-E2 R3-S1-R35-E2-F1: https://www.comscore.com/Insights/Presentations-and-Whitepapers/2026/2026-Football-Kickoff-Guide；https://www.comscore.com/Insights/Presentations-and-Whitepapers/2026/2026-Fall-and-Halloween-Guide（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>S1-R35-E1 规则：R3-S1-R35-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）、留出反例 1&lt;3）；链接 可打开（200，标题「Blog - Comscore, Inc.」）
-S1-R35-E2 规则：R3-S1-R35-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）、留出反例 1&lt;3）；链接 可打开（200，标题「Presentations and Whitepapers - Comscore, Inc.」）</t>
+          <t>S1-R35-E1 规则：R3-S1-R35-E1-F1 部分验证（候选）（机械门未通过：留出与归纳/回归重叠）；链接 可打开（200，标题「Blog - Comscore, Inc.」）
+S1-R35-E2 R3-S1-R35-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP4/FP0/FN0/TN4；覆盖检查：列表 19 个、sitemap 同结构 0 个全部匹配
+S1-R35-E2 规则：R3-S1-R35-E2-F1 已验证；链接 可打开（200，标题「Presentations and Whitepapers - Comscore, Inc.」）</t>
         </is>
       </c>
       <c r="G35" s="3" t="inlineStr">
@@ -2152,6 +2242,7 @@
       <c r="B39" s="4" t="inlineStr">
         <is>
           <t>^https://www\.gwi\.com/blog/[a-z0-9-]+$
+^https://www\.gwi\.com/blog/tag/[a-z-]+$
 ^https://www\.gwi\.com/case\-studies/[a-z0-9-]+$</t>
         </is>
       </c>
@@ -2160,7 +2251,7 @@
           <t>S1-R39-E1: https://www.gwi.com/reports
   其余 108 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E1.txt
 S1-R39-E2: https://www.gwi.com/blog
-  其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E2.txt
+  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E2.txt
 S1-R39-E3: https://www.gwi.com/case-studies
   其余 8 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E3.txt</t>
         </is>
@@ -2168,6 +2259,7 @@
       <c r="D39" s="3" t="inlineStr">
         <is>
           <t>S1-R39-E2 R3-S1-R39-E2-F1: https://www.gwi.com/blog/brand-purpose；https://www.gwi.com/blog/2025-predictions-vs-reality（已落地核验 200，公开访问，2026-10-26）
+S1-R39-E2 R3-S1-R39-E2-F2: https://www.gwi.com/blog/tag/consumer-behavior；https://www.gwi.com/blog/tag/data-journalism（已落地核验 200，公开访问，2026-10-26）
 S1-R39-E3 R3-S1-R39-E3-F1: https://www.gwi.com/case-studies/conde-nast；https://www.gwi.com/case-studies/barefoot-proximity（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
@@ -2180,7 +2272,8 @@
         <is>
           <t>S1-R39-E1 规则：R3-S1-R39-E1-F1 部分验证（候选）（机械门未通过：标注测试有失败（留出 FN0/FP0））；链接 可打开（200，标题「Reports - Resources, Marketing Infographics &amp; Guid」）
 S1-R39-E2 R3-S1-R39-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 21 个、sitemap 同结构 458 个全部匹配
-S1-R39-E2 规则：R3-S1-R39-E2-F1 已验证；R3-S1-R39-E2-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Digital &amp; Social Trends, Charts, Consumer Data &amp; S」）
+S1-R39-E2 R3-S1-R39-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
+S1-R39-E2 规则：R3-S1-R39-E2-F1 已验证；R3-S1-R39-E2-F2 已验证；链接 可打开（200，标题「Digital &amp; Social Trends, Charts, Consumer Data &amp; S」）
 S1-R39-E3 R3-S1-R39-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP2/FP0/FN0/TN5；覆盖检查：列表 38 个、sitemap 同结构 35 个全部匹配
 S1-R39-E3 规则：R3-S1-R39-E3-F1 已验证；链接 可打开（200，标题「Case Studies - How Agencies, Businesses &amp; Brands u」）</t>
         </is>
@@ -2258,30 +2351,33 @@
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>^https://interbrand\.com/thinking/[a-z-]+/$</t>
+          <t>^https://interbrand\.com/best\-global\-brands/global/[a-z0-9-]+/$
+^https://interbrand\.com/thinking/[a-z-]+/$</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
           <t>S1-R41-E1: https://interbrand.com/best-global-brands/
-  其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R41-E1.txt
+  其余 3 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R41-E1.txt
 S1-R41-E2: https://interbrand.com/thinking/
   其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R41-E2.txt</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>S1-R41-E2 R3-S1-R41-E2-F1: https://interbrand.com/thinking/design-leader-fura-johannesdottir-global-chief-creative-officer-at-interbrand/；https://interbrand.com/thinking/allianz-brand-trust/（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R41-E1 R3-S1-R41-E1-F1: https://interbrand.com/best-global-brands/global/ebay/；https://interbrand.com/best-global-brands/global/apple/（已落地核验 200，公开访问，2026-10-26）
+S1-R41-E2 R3-S1-R41-E2-F1: https://interbrand.com/thinking/design-leader-fura-johannesdottir-global-chief-creative-officer-at-interbrand/；https://interbrand.com/thinking/allianz-brand-trust/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>S1-R41-E1 规则：R3-S1-R41-E1-F1 部分验证（候选）（机械门未通过：留出反例 0&lt;3）；链接 可打开（200，标题「Best Global Brands - Interbrand」）
+          <t>S1-R41-E1 R3-S1-R41-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 10 个、sitemap 同结构 105 个全部匹配
+S1-R41-E1 规则：R3-S1-R41-E1-F1 已验证；链接 可打开（200，标题「Best Global Brands - Interbrand」）
 S1-R41-E2 R3-S1-R41-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 4 个、sitemap 同结构 10 个全部匹配
 S1-R41-E2 规则：R3-S1-R41-E2-F1 已验证；链接 可打开（200，标题「Thinking - Interbrand」）</t>
         </is>
@@ -2294,7 +2390,7 @@
       </c>
       <c r="H41" s="3" t="inlineStr">
         <is>
-          <t>S1-R41-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /best-global-brands/ 下家族 1 个、成员 10；前缀外同站链接 1、文件 1；sitemap 中同结构但不在列表的 URL：F1=95
+          <t>S1-R41-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /best-global-brands/ 下家族 1 个、成员 10；前缀外同站链接 1、文件 1；sitemap 中同结构但不在列表的 URL：F1=95
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R41-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /thinking/ 下家族 1 个、成员 4；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=6
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -2465,9 +2561,9 @@
       <c r="C45" s="3" t="inlineStr">
         <is>
           <t>S1-R45-E1: https://yougov.com/content/economy
-  其余 40 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R45-E1.txt
+  其余 41 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R45-E1.txt
 S1-R45-E2: https://yougov.com/content/consumer
-  其余 2669 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R45-E2.txt
+  其余 2726 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R45-E2.txt
 S1-R45-E3: https://yougov.com/reports
   其余 16 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R45-E3.txt
 S1-R45-E4: https://yougov.com/business/sectors/consumer
@@ -2503,10 +2599,10 @@
       </c>
       <c r="H45" s="3" t="inlineStr">
         <is>
-          <t>S1-R45-E1: 部分：Load more 点到按钮消失：接口 hits=1016，页面内容链接 1,015，差 1 未解释
+          <t>S1-R45-E1: 完整：Load more 点到按钮消失时页面有 1,015 条；页面在接口还有 1 条时隐藏了按钮。用页面自身的只读接口取 offset=1015 补到 1 条（id 11767，已落地 200），合计 1,016 = 接口 hits
   完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /content/economy/ 下家族 0 个、成员 0；前缀外同站链接 40、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：完整（本次筛选条件下）：浏览器渲染并点击 button.load-more（CSS 隐藏 Cookie 弹层，未点同意）；组件只读 GET api-test.yougov.com/public-content/content（limit=35，offset 递增）；接口 hits=1016，点击 28 次后按钮消失，页面取得 1,015 个内容链接（articles 899、reports 92、case-studies 13、guides 8、events 3），差 1 未解释；续跑见 output/round3/queue.json
-S1-R45-E2: 部分：Load more 点到按钮消失（76 次）：接口 hits=2717，页面内容链接 2,660，差 57 未解释
+S1-R45-E2: 完整：Load more 点到按钮消失时页面有 2,660 条；页面在接口还有 57 条时隐藏了按钮。用页面自身的只读接口取 offset=2660、2695 补到 57 条（全部落地 200），合计 2,717 = 接口 hits
   完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 77 轮、点击加载更多 75 次、渲染后链接 2893；前缀 /content/consumer/ 下家族 0 个、成员 0；前缀外同站链接 2669、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：部分：浏览器渲染并点击 button.load-more（CSS 隐藏 Cookie 弹层，未点同意）；组件只读 GET api-test.yougov.com/public-content/content（limit=35，offset 递增）；接口 hits=2717，本批 45 轮取得约 1,575 个内容链接（articles 1,300、reports 229…），剩余约 1,142 条待续跑；续跑见 output/round3/queue.json
 S1-R45-E3: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /reports/ 下家族 1 个、成员 36；前缀外同站链接 16、文件 0；sitemap 中同结构但不在列表的 URL：F1=429
@@ -2646,22 +2742,31 @@
           <t>https://www.bain.com/insights/</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.bain\.com/insights/[a-zA-Z0-9_-]+/$</t>
+        </is>
+      </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
           <t>S1-R48-E1: https://www.bain.com/insights/
-  其余 40 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R48-E1.txt</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr"/>
+  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R48-E1.txt</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>S1-R48-E1 R3-S1-R48-E1-F1: https://www.bain.com/insights/2020-year-in-review-the-surprising-resilience-m-and-a-report-2021/；https://www.bain.com/insights/black-friday-2026-sales-forecast-infographic/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
         <is>
-          <t>S1-R48-E1 规则：R3-S1-R48-E1-F1 部分验证（候选）（机械门未通过：有正例未完成落地身份核验）；链接 可打开（200，标题「Bain Insights &amp; Publications | Bain &amp; Company」）</t>
+          <t>S1-R48-E1 R3-S1-R48-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 21 个、sitemap 同结构 6295 个全部匹配
+S1-R48-E1 规则：R3-S1-R48-E1-F1 已验证；链接 可打开（200，标题「Bain Insights &amp; Publications | Bain &amp; Company」）</t>
         </is>
       </c>
       <c r="G48" s="3" t="inlineStr">
@@ -2671,7 +2776,7 @@
       </c>
       <c r="H48" s="3" t="inlineStr">
         <is>
-          <t>S1-R48-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 1 次、渲染后链接 250；前缀 /insights/ 下家族 2 个、成员 24；前缀外同站链接 16、文件 0；sitemap 中同结构但不在列表的 URL：F1=6291
+          <t>S1-R48-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 1 次、渲染后链接 250；前缀 /insights/ 下家族 2 个、成员 24；前缀外同站链接 16、文件 0；sitemap 中同结构但不在列表的 URL：F1=6291
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -2725,7 +2830,7 @@
       </c>
       <c r="H49" s="3" t="inlineStr">
         <is>
-          <t>S1-R49-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /global/en/insights/ 下家族 3 个、成员 32；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=1098、F2=36
+          <t>S1-R49-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /global/en/insights/ 下家族 3 个、成员 32；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=1098、F2=36
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -2751,7 +2856,7 @@
           <t>S1-R50-E1: https://www.forrester.com/b2b-marketing/
   其余 39 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R50-E1.txt
 S1-R50-E2: https://www.forrester.com/b2c-marketing/
-  其余 33 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R50-E2.txt
+  其余 34 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R50-E2.txt
 S1-R50-E3: https://www.forrester.com/blogs/category/b2b-research/
   其余 1324 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R50-E3.txt
 S1-R50-E4: https://www.forrester.com/blogs/category/b2b-research/page/2/
@@ -2784,12 +2889,13 @@
         <is>
           <t>S1-R50-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 254；前缀 /b2b-marketing/ 下家族 0 个、成员 0；前缀外同站链接 37、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R50-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 242；前缀 /b2c-marketing/ 下家族 0 个、成员 0；前缀外同站链接 33、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R50-E3: 部分：页面 More posts 点到按钮消失，列表 1,221 篇，全部在 WP REST 1,222 篇内；未在列表出现的 1 篇已定位（id 122415，2018-05-09）；分类计数 1,287 与公开 1,222 差 65 未解释
+S1-R50-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 242；前缀 /b2c-marketing/ 下家族 0 个、成员 0；前缀外同站链接 33、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R50-E3: 完整：页面 More posts 点到按钮消失，列表 1,221 篇，全部在 WP REST 公开文章 1,222 篇（X-WP-Total）内；未在列表出现的 1 篇已定位（id 122415，2018-05-09）。分类计数 1,287 是 WordPress 内部计数，可能含非公开文章，公开接口无法核实，不作为对账总数
   完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 63 轮、点击加载更多 61 次、渲染后链接 3369；前缀 /blogs/category/b2b-research/ 下家族 0 个、成员 0；前缀外同站链接 1324、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：部分：根因已查清——列表页底部 More posts 调用 POST go.forrester.com/wp-admin/admin-ajax.php action=loadposts&amp;page=N&amp;category=b2b-research，data-pages=62；/page/N/ 地址的静态正文不随页码变化。成员集合经 WP REST GET（categories=50231）取得 1,222 篇（X-WP-Total=1222，与 62 页×20 吻合），首页 16 篇全部在内；分类计数 1,287 与公开文章数差 65 未解释；loadposts POST 本轮未执行（权限拦截）；续跑见 output/round3/queue.json
-S1-R50-E4: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 20 轮、点击加载更多 20 次、渲染后链接 1331；前缀 /blogs/category/b2b-research/page/2/ 下家族 0 个、成员 0；前缀外同站链接 497、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+S1-R50-E4: 完整：/page/2/ 与 S1-R50-E3 是同一栏目、同一列表（服务端忽略页码），成员与对账同 S1-R50-E3
+  部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 20 轮、点击加载更多 20 次、渲染后链接 1331；前缀 /blogs/category/b2b-research/page/2/ 下家族 0 个、成员 0；前缀外同站链接 497、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：部分：/page/2/ 静态返回与第 1 页相同的 16 篇（30/30 链接一致），JS 变量 current_page=2，仅影响 More posts 起始页；同栏目成员见 S1-R50-E3；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -2887,7 +2993,13 @@
 https://www.pewresearch.org/topic/economy-work/business-workplace/</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr"/>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.pewresearch\.org/topic/economy\-work/page/[0-9]+/$
+^https://www\.pewresearch\.org/topic/internet\-technology/[a-z-]+/[a-z0-9-]+/$
+^https://www\.pewresearch\.org/topic/news\-habits\-media/[a-z-]+/[a-z0-9-]+/$</t>
+        </is>
+      </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
           <t>S1-R52-E1: https://www.pewresearch.org/topic/economy-work/
@@ -2895,22 +3007,31 @@
 S1-R52-E2: https://www.pewresearch.org/topic/internet-technology/
   其余 21 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R52-E2.txt
 S1-R52-E3: https://www.pewresearch.org/topic/news-habits-media/
-  其余 41 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R52-E3.txt
+  其余 42 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R52-E3.txt
 S1-R52-E4: https://www.pewresearch.org/topic/economy-work/business-workplace/
   其余 85 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R52-E4.txt</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>S1-R52-E1 R3-S1-R52-E1-F1: https://www.pewresearch.org/topic/economy-work/page/161/；https://www.pewresearch.org/topic/economy-work/page/163/（已落地核验 200，公开访问，2026-10-26）
+S1-R52-E2 R3-S1-R52-E2-F1: https://www.pewresearch.org/topic/internet-technology/emerging-technology/bots/；https://www.pewresearch.org/topic/internet-technology/emerging-technology/artificial-intelligence/（已落地核验 200，公开访问，2026-10-26）
+S1-R52-E3 R3-S1-R52-E3-F1: https://www.pewresearch.org/topic/news-habits-media/media-society/freedom-of-the-press/；https://www.pewresearch.org/topic/news-habits-media/news-media-trends/local-news/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 链接保留</t>
         </is>
       </c>
       <c r="F52" s="3" t="inlineStr">
         <is>
-          <t>S1-R52-E1 规则：无规则；链接 可打开（200，标题「Economy &amp; Work - Research and data from Pew Resear」）
-S1-R52-E2 规则：无规则；链接 可打开（200，标题「Internet &amp; Technology - Research and data from Pew」）
-S1-R52-E3 规则：无规则；链接 可打开（200，标题「News Habits &amp; Media - Research and data from Pew R」）
+          <t>S1-R52-E1 R3-S1-R52-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP5/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
+S1-R52-E1 规则：R3-S1-R52-E1-F1 已验证；链接 可打开（200，标题「Economy &amp; Work - Research and data from Pew Resear」）
+S1-R52-E2 R3-S1-R52-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 4 个、sitemap 同结构 28 个全部匹配
+S1-R52-E2 规则：R3-S1-R52-E2-F1 已验证；链接 可打开（200，标题「Internet &amp; Technology - Research and data from Pew」）
+S1-R52-E3 R3-S1-R52-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 5 个、sitemap 同结构 12 个全部匹配
+S1-R52-E3 规则：R3-S1-R52-E3-F1 已验证；链接 可打开（200，标题「News Habits &amp; Media - Research and data from Pew R」）
 S1-R52-E4 规则：无规则；链接 可打开（200，标题「Business &amp; Workplace - Research and data from Pew 」）</t>
         </is>
       </c>
@@ -2924,11 +3045,11 @@
       </c>
       <c r="H52" s="3" t="inlineStr">
         <is>
-          <t>S1-R52-E1: 完整（枚举结束，无独立全集对账）：静态请求 6 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 129；前缀 /topic/economy-work/ 下家族 0 个、成员 0；前缀外同站链接 30、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R52-E2: 完整（枚举结束，无独立全集对账）：静态请求 4 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 145；前缀 /topic/internet-technology/ 下家族 0 个、成员 0；前缀外同站链接 21、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R52-E3: 完整（枚举结束，无独立全集对账）：静态请求 7 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 147；前缀 /topic/news-habits-media/ 下家族 0 个、成员 0；前缀外同站链接 41、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+          <t>S1-R52-E1: 完整（枚举结束，无独立全集对账）：静态请求 6 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 129；前缀 /topic/economy-work/ 下家族 1 个、成员 3；前缀外同站链接 30、文件 0；sitemap 中同结构但不在列表的 URL：F1=0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R52-E2: 部分：静态请求 4 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 145；前缀 /topic/internet-technology/ 下家族 1 个、成员 4；前缀外同站链接 21、文件 0；sitemap 中同结构但不在列表的 URL：F1=27；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R52-E3: 部分：静态请求 7 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 147；前缀 /topic/news-habits-media/ 下家族 1 个、成员 5；前缀外同站链接 41、文件 0；sitemap 中同结构但不在列表的 URL：F1=11；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R52-E4: 完整（枚举结束，无独立全集对账）：静态请求 15 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 120；前缀 /topic/economy-work/business-workplace/ 下家族 0 个、成员 0；前缀外同站链接 85、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -2951,7 +3072,8 @@
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.idc\.com/data\-analytics/[a-z-]+/?$
+          <t>^https://www\.idc\.com/research/[a-z-]+/?$
+^https://www\.idc\.com/data\-analytics/[a-z-]+/?$
 ^https://www\.idc\.com/quanta/[a-z-]+/$
 ^https://www\.idc\.com/resource\-center/blog/[a-z0-9%-]+/$
 ^https://www\.idc\.com/resource\-center/[a-z0-9-]+/$</t>
@@ -2960,7 +3082,7 @@
       <c r="C53" s="3" t="inlineStr">
         <is>
           <t>S1-R53-E1: https://www.idc.com/research/
-  其余 12 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R53-E1.txt
+  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R53-E1.txt
 S1-R53-E2: https://www.idc.com/data-analytics/
   其余 8 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R53-E2.txt
 S1-R53-E3: https://www.idc.com/quanta/
@@ -2971,7 +3093,8 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>S1-R53-E2 R3-S1-R53-E2-F1: https://www.idc.com/data-analytics/news/；https://www.idc.com/data-analytics/black-book（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R53-E1 R3-S1-R53-E1-F1: https://www.idc.com/research/investment-research；https://www.idc.com/research/digital-business（已落地核验 200，公开访问，2026-10-26）
+S1-R53-E2 R3-S1-R53-E2-F1: https://www.idc.com/data-analytics/news/；https://www.idc.com/data-analytics/black-book（已落地核验 200，公开访问，2026-10-26）
 S1-R53-E3 R3-S1-R53-E3-F1: https://www.idc.com/quanta/book-a-demo/；https://www.idc.com/quanta/tech-leader/（已落地核验 200，公开访问，2026-10-26）
 S1-R53-E4 R3-S1-R53-E4-F1: https://www.idc.com/resource-center/blog/%e6%9c%ba%e5%99%a8%e4%ba%ba%e6%ad%a3%e5%9c%a8%e8%bf%9b%e5%8c%96-2026%e5%b9%b4%e4%b8%ad%e5%9b%bd%e6%9c%ba%e5%99%a8%e4%ba%ba%e4%b8%8e%e5%85%b7%e8%ba%ab%e6%99%ba/；https://www.idc.com/resource-center/blog/ai-is-short-of-capacity-not-demand/（已落地核验 200，公开访问，2026-10-26）
 S1-R53-E4 R3-S1-R53-E4-F2: https://www.idc.com/resource-center/ai-hub/；https://www.idc.com/resource-center/blog/（已落地核验 200，公开访问，2026-10-26）</t>
@@ -2979,12 +3102,13 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 正则+链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 正则+链接保留</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>S1-R53-E1 规则：R3-S1-R53-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「IDC.com - Research - Overview」）
+          <t>S1-R53-E1 R3-S1-R53-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN5；覆盖检查：列表 6 个、sitemap 同结构 6 个全部匹配
+S1-R53-E1 规则：R3-S1-R53-E1-F1 已验证；链接 可打开（200，标题「IDC.com - Research - Overview」）
 S1-R53-E2 R3-S1-R53-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP1/FP0/FN0/TN5；覆盖检查：列表 6 个、sitemap 同结构 7 个全部匹配
 S1-R53-E2 规则：R3-S1-R53-E2-F1 已验证；链接 可打开（200，标题「IDC - Data Analytics - Home」）
 S1-R53-E3 R3-S1-R53-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP2/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 5 个全部匹配
@@ -3004,7 +3128,7 @@
       </c>
       <c r="H53" s="3" t="inlineStr">
         <is>
-          <t>S1-R53-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 1 个、成员 6；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=6
+          <t>S1-R53-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 1 个、成员 6；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=6
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R53-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /data-analytics/ 下家族 1 个、成员 6；前缀外同站链接 8、文件 0；sitemap 中同结构但不在列表的 URL：F1=7
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -3150,7 +3274,7 @@
       <c r="C62" s="3" t="inlineStr">
         <is>
           <t>S1-R62-E1: https://ads.tiktok.com/creative/creativeCenter
-  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R62-E1.txt</t>
+  其余 10 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R62-E1.txt</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr"/>
@@ -3161,7 +3285,7 @@
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>S1-R62-E1 规则：无规则；链接 可打开（200，标题「TikTok One Creative Suite」）</t>
+          <t>S1-R62-E1 规则：R3-S1-R62-E1-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「TikTok One Creative Suite」）</t>
         </is>
       </c>
       <c r="G62" s="3" t="inlineStr">
@@ -3171,7 +3295,7 @@
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
-          <t>S1-R62-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 0；前缀 /creative/creativeCenter/ 下家族 0 个、成员 0；前缀外同站链接 6、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+          <t>S1-R62-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 0；前缀 /creative/creativeCenter/ 下家族 1 个、成员 3；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -3293,8 +3417,8 @@
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>S1-R65-E1 R3-S1-R65-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN4；覆盖检查：列表 19 个、sitemap 同结构 0 个全部匹配
-S1-R65-E1 R3-S1-R65-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN4；覆盖检查：列表 8 个、sitemap 同结构 0 个全部匹配
+          <t>S1-R65-E1 R3-S1-R65-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN6；覆盖检查：列表 19 个、sitemap 同结构 0 个全部匹配
+S1-R65-E1 R3-S1-R65-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN6；覆盖检查：列表 8 个、sitemap 同结构 0 个全部匹配
 S1-R65-E1 规则：R3-S1-R65-E1-F1 已验证；R3-S1-R65-E1-F2 已验证；链接 可打开（200，标题「Marketing &amp; Advertising Blog | LinkedIn for Market」）</t>
         </is>
       </c>
@@ -4083,6 +4207,8 @@
         <is>
           <t>^https://www\.dandad\.org/work/annual\-2026/[a-z0-9-]+/[a-z0-9íüē-]+$
 ^https://www\.dandad\.org/insights/[a-z-]+/[a-zA-Z0-9ü-]+$
+^https://www\.dandad\.org/insights/[a-z-]+$
+^https://www\.dandad\.org/insights/case\-studies\-and\-partnerships/[a-z-]+$
 ^https://www\.dandad\.org/work/d\-ad\-awards\-archive/[a-z0-9_ßàáâãäåæçèéêíðñòóôöøúüāđēīņōœśšžǎǐ我水-]+$</t>
         </is>
       </c>
@@ -4091,9 +4217,9 @@
           <t>S1-R86-E1: https://www.dandad.org/work/annual-2026/
   其余 66 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E1.txt
 S1-R86-E2: https://www.dandad.org/insights
-  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E2.txt
+  其余 15 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E2.txt
 S1-R86-E3: https://www.dandad.org/insights/case-studies-and-partnerships
-  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E3.txt
+  其余 9 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E3.txt
 S1-R86-E4: https://www.dandad.org/work/d-ad-awards-archive
   其余 11 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R86-E4.txt
 S1-R86-E5: https://www.dandad.org/subjects/case-study
@@ -4104,12 +4230,14 @@
         <is>
           <t>S1-R86-E1 R3-S1-R86-E1-F1: https://www.dandad.org/work/annual-2026/judges-curations/curation-by-astrid-stavro-magazine-newspaper-design；https://www.dandad.org/work/annual-2026/behind-the-work/how-bad-bunnys-interactive-album-teaser-bridged-local-and-global-fandoms（已落地核验 200，公开访问，2026-10-26）
 S1-R86-E2 R3-S1-R86-E2-F1: https://www.dandad.org/insights/awards/amex-small-business-saturday-case-study-insights；https://www.dandad.org/insights/awards/dad-awards-2026-watch-our-webinars-on-whats-new-and-how-to-enter（已落地核验 200，公开访问，2026-10-26）
+S1-R86-E2 R3-S1-R86-E2-F2: https://www.dandad.org/insights/awards；https://www.dandad.org/insights/case-studies-and-partnerships（已落地核验 200，公开访问，2026-10-26）
+S1-R86-E3 R3-S1-R86-E3-F1: https://www.dandad.org/insights/case-studies-and-partnerships/how-creativity-and-innovation-drive-impact；https://www.dandad.org/insights/case-studies-and-partnerships/glimpse-masterclass-case-study（已落地核验 200，公开访问，2026-10-26）
 S1-R86-E4 R3-S1-R86-E4-F1: https://www.dandad.org/work/d-ad-awards-archive/ariel-share-the-load；https://www.dandad.org/work/d-ad-awards-archive/100-words-for-water-a-projective-ecosocial-vocabulary（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 正则+链接保留；E3 链接保留；E4 正则+链接保留；E5 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 正则+链接保留；E5 链接保留</t>
         </is>
       </c>
       <c r="F86" s="3" t="inlineStr">
@@ -4117,8 +4245,10 @@
           <t>S1-R86-E1 R3-S1-R86-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 40 个、sitemap 同结构 49 个全部匹配
 S1-R86-E1 规则：R3-S1-R86-E1-F1 已验证；R3-S1-R86-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「D&amp;AD Annual 2026」）
 S1-R86-E2 R3-S1-R86-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 46 个、sitemap 同结构 409 个全部匹配
-S1-R86-E2 规则：R3-S1-R86-E2-F1 已验证；R3-S1-R86-E2-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Insights」）
-S1-R86-E3 规则：R3-S1-R86-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Case studies and partnerships | Insights」）
+S1-R86-E2 R3-S1-R86-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 4 个、sitemap 同结构 4 个全部匹配
+S1-R86-E2 规则：R3-S1-R86-E2-F1 已验证；R3-S1-R86-E2-F2 已验证；链接 可打开（200，标题「Insights」）
+S1-R86-E3 R3-S1-R86-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP2/FP0/FN0/TN5；覆盖检查：列表 10 个、sitemap 同结构 10 个全部匹配
+S1-R86-E3 规则：R3-S1-R86-E3-F1 已验证；链接 可打开（200，标题「Case studies and partnerships | Insights」）
 S1-R86-E4 R3-S1-R86-E4-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 12 个、sitemap 同结构 21878 个全部匹配
 S1-R86-E4 规则：R3-S1-R86-E4-F1 已验证；链接 可打开（200，标题「D&amp;AD Awards archive」）
 S1-R86-E5 规则：无规则；链接 可打开（200，标题「Case Study」）</t>
@@ -4163,7 +4293,8 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.demandcurve\.com/frontier\-library/[a-z-]+$</t>
+          <t>^https://www\.demandcurve\.com/frontier\-library/[a-z-]+$
+^https://gp\.demandcurve\.com/blog/[a-z-]+$</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -4173,17 +4304,18 @@
 S1-R87-E2: https://gp.demandcurve.com/resources
   其余 22 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R87-E2.txt
 S1-R87-E3: https://gp.demandcurve.com/blog
-  其余 60 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R87-E3.txt</t>
+  其余 22 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R87-E3.txt</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>S1-R87-E1 R3-S1-R87-E1-F1: https://www.demandcurve.com/frontier-library/analytics；https://www.demandcurve.com/frontier-library/ai-growth（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R87-E1 R3-S1-R87-E1-F1: https://www.demandcurve.com/frontier-library/analytics；https://www.demandcurve.com/frontier-library/ai-growth（已落地核验 200，公开访问，2026-10-26）
+S1-R87-E3 R3-S1-R87-E3-F1: https://gp.demandcurve.com/blog/cold-email-marketing；https://gp.demandcurve.com/blog/copywriting-examples（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 链接保留；E3 链接保留</t>
+          <t>E1 正则+链接保留；E2 链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F87" s="3" t="inlineStr">
@@ -4191,7 +4323,8 @@
           <t>S1-R87-E1 R3-S1-R87-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP2/FP0/FN0/TN5；覆盖检查：列表 11 个、sitemap 同结构 13 个全部匹配
 S1-R87-E1 规则：R3-S1-R87-E1-F1 已验证；链接 可打开（200，标题「Growth Content Library | The Frontier by Demand Cu」）
 S1-R87-E2 规则：无规则；链接 可打开（200，标题「Demand Curve Resources」）
-S1-R87-E3 规则：R3-S1-R87-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Growth Marketing Blog by Demand Curve」）</t>
+S1-R87-E3 R3-S1-R87-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN5；覆盖检查：列表 38 个、sitemap 同结构 38 个全部匹配
+S1-R87-E3 规则：R3-S1-R87-E3-F1 已验证；链接 可打开（200，标题「Growth Marketing Blog by Demand Curve」）</t>
         </is>
       </c>
       <c r="G87" s="3" t="inlineStr">
@@ -4248,7 +4381,7 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>S1-R88-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 44；前缀 /omnichannel-study/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+          <t>S1-R88-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 44；前缀 /omnichannel-study/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；页面上没有可枚举的标准链接（a[href]），内容可能由脚本组件渲染
   第 2 轮人工复核：部分：入口静态首轮 1 页（2189 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -4300,7 +4433,7 @@
 S1-R89-E2 R3-S1-R89-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 66 个、sitemap 同结构 5213 个全部匹配
 S1-R89-E2 R3-S1-R89-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 36 个、sitemap 同结构 847 个全部匹配
 S1-R89-E2 规则：R3-S1-R89-E2-F1 已验证；R3-S1-R89-E2-F2 已验证；第 2 轮：无规则；链接 可打开（200，标题「Insights — Greenbook」）
-S1-R89-E3 规则：R3-S1-R89-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则；链接 可打开（200，标题「GRIT — Greenbook」）</t>
+S1-R89-E3 规则：R3-S1-R89-E3-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则；链接 可打开（200，标题「GRIT — Greenbook」）</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -4335,22 +4468,31 @@
           <t>https://growth.design/case-studies</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr"/>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>^https://growth\.design/case\-studies/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
           <t>S1-R90-E1: https://growth.design/case-studies
-  其余 52 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R90-E1.txt</t>
-        </is>
-      </c>
-      <c r="D90" s="3" t="inlineStr"/>
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R90-E1.txt</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>S1-R90-E1 R3-S1-R90-E1-F1: https://growth.design/case-studies/adobe-trial-ux；https://growth.design/case-studies/labor-perception-bias（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>S1-R90-E1 规则：R3-S1-R90-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「52 UX Case Studies To Improve Your Product Skills 」）</t>
+          <t>S1-R90-E1 R3-S1-R90-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN4；覆盖检查：列表 52 个、sitemap 同结构 52 个全部匹配
+S1-R90-E1 规则：R3-S1-R90-E1-F1 已验证；链接 可打开（200，标题「52 UX Case Studies To Improve Your Product Skills 」）</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -4539,28 +4681,40 @@
 https://marketingexamples.com/copywriting</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr"/>
+      <c r="B95" s="4" t="inlineStr">
+        <is>
+          <t>^https://marketingexamples\.com/social/[a-z-]+$
+^https://marketingexamples\.com/copywriting/[a-z-]+$</t>
+        </is>
+      </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
           <t>S1-R95-E2: https://marketingexamples.com/inspiration
   其余 21 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R95-E2.txt
 S1-R95-E3: https://marketingexamples.com/social
-  其余 38 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R95-E3.txt
+  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R95-E3.txt
 S1-R95-E4: https://marketingexamples.com/copywriting
-  其余 33 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R95-E4.txt</t>
-        </is>
-      </c>
-      <c r="D95" s="3" t="inlineStr"/>
+  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R95-E4.txt</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>S1-R95-E3 R3-S1-R95-E3-F1: https://marketingexamples.com/social/calvin-klein；https://marketingexamples.com/social/ama（已落地核验 200，公开访问，2026-10-26）
+S1-R95-E4 R3-S1-R95-E4-F1: https://marketingexamples.com/copywriting/adjectives；https://marketingexamples.com/copywriting/bou（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>E2 链接保留；E3 链接保留；E4 链接保留；E1 host免提</t>
+          <t>E2 链接保留；E3 正则+链接保留；E4 正则+链接保留；E1 host免提</t>
         </is>
       </c>
       <c r="F95" s="3" t="inlineStr">
         <is>
           <t>S1-R95-E2 规则：无规则；链接 可打开（200，标题「Copywriting Examples - The world's best copy. In o」）
-S1-R95-E3 规则：R3-S1-R95-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Social Marketing Examples」）
-S1-R95-E4 规则：R3-S1-R95-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Copywriting Marketing Examples」）</t>
+S1-R95-E3 R3-S1-R95-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP4/FP0/FN0/TN5；覆盖检查：列表 19 个、sitemap 同结构 19 个全部匹配
+S1-R95-E3 规则：R3-S1-R95-E3-F1 已验证；链接 可打开（200，标题「Social Marketing Examples」）
+S1-R95-E4 R3-S1-R95-E4-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP3/FP0/FN0/TN5；覆盖检查：列表 14 个、sitemap 同结构 14 个全部匹配
+S1-R95-E4 规则：R3-S1-R95-E4-F1 已验证；链接 可打开（200，标题「Copywriting Marketing Examples」）</t>
         </is>
       </c>
       <c r="G95" s="3" t="inlineStr">
@@ -4696,7 +4850,7 @@
       <c r="F99" s="3" t="inlineStr">
         <is>
           <t>S1-R99-E1 R3-S1-R99-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 10 个、sitemap 同结构 285 个全部匹配
-S1-R99-E1 规则：R3-S1-R99-E1-F1 已验证；R3-S1-R99-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The Reforge Blog | Reforge」）</t>
+S1-R99-E1 规则：R3-S1-R99-E1-F1 已验证；R3-S1-R99-E1-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The Reforge Blog | Reforge」）</t>
         </is>
       </c>
       <c r="G99" s="3" t="inlineStr">
@@ -4833,7 +4987,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>S1-R103-E1 R3-S1-R103-E1-F2: https://www.oneclub.org/awards/theoneshow/-award/21921/thick-fine/；https://www.oneclub.org/awards/theoneshow/-award/63830/breastmilk-money/（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R103-E1 R3-S1-R103-E1-F2: https://www.oneclub.org/awards/theoneshow/-award/1131/bucket/；https://www.oneclub.org/awards/theoneshow/-award/63830/breastmilk-money/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
@@ -4843,7 +4997,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>S1-R103-E1 R3-S1-R103-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 50 个、sitemap 同结构 16529 个全部匹配
+          <t>S1-R103-E1 R3-S1-R103-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 50 个、sitemap 同结构 34054 个全部匹配
 S1-R103-E1 规则：R3-S1-R103-E1-F2 已验证；链接 可打开（200，标题「One Show | Awards Archive | 2026」）</t>
         </is>
       </c>
@@ -4854,7 +5008,7 @@
       </c>
       <c r="H103" s="3" t="inlineStr">
         <is>
-          <t>S1-R103-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /awards/theoneshow/ 下家族 2 个、成员 354；前缀外同站链接 19、文件 0；sitemap 中同结构但不在列表的 URL：F2=16479
+          <t>S1-R103-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /awards/theoneshow/ 下家族 2 个、成员 354；前缀外同站链接 19、文件 0；sitemap 中同结构但不在列表的 URL：F2=34004
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -4875,13 +5029,15 @@
       </c>
       <c r="B104" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.thinkbox\.tv/news\-and\-opinion/[a-z0-9-]+$</t>
+          <t>^https://www\.thinkbox\.tv/research/[a-z-]+/[a-z0-9-]+$
+^https://www\.thinkbox\.tv/research/[a-z-]+$
+^https://www\.thinkbox\.tv/news\-and\-opinion/[a-z0-9-]+$</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
         <is>
           <t>S1-R104-E1: https://www.thinkbox.tv/research
-  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R104-E1.txt
+  其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R104-E1.txt
 S1-R104-E2: https://www.thinkbox.tv/case-studies
   其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R104-E2.txt
 S1-R104-E3: https://www.thinkbox.tv/news-and-opinion
@@ -4890,17 +5046,21 @@
       </c>
       <c r="D104" s="3" t="inlineStr">
         <is>
-          <t>S1-R104-E3 R3-S1-R104-E3-F1: https://www.thinkbox.tv/news-and-opinion/cflight-your-questions-answered；https://www.thinkbox.tv/news-and-opinion/events（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R104-E1 R3-S1-R104-E1-F1: https://www.thinkbox.tv/research/charts-on-film/media-signalling；https://www.thinkbox.tv/research/nickable-charts/addressable（已落地核验 200，公开访问，2026-10-26）
+S1-R104-E1 R3-S1-R104-E1-F2: https://www.thinkbox.tv/research/nickable-charts；https://www.thinkbox.tv/research/charts-on-film（已落地核验 200，公开访问，2026-10-26）
+S1-R104-E3 R3-S1-R104-E3-F1: https://www.thinkbox.tv/news-and-opinion/cflight-your-questions-answered；https://www.thinkbox.tv/news-and-opinion/events（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 正则+链接保留</t>
+          <t>E1 正则+链接保留；E2 链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
         <is>
-          <t>S1-R104-E1 规则：无规则；链接 可打开（200，标题「Research」）
+          <t>S1-R104-E1 R3-S1-R104-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN7；覆盖检查：列表 43 个、sitemap 同结构 37 个全部匹配
+S1-R104-E1 R3-S1-R104-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 4 个、sitemap 同结构 4 个全部匹配
+S1-R104-E1 规则：R3-S1-R104-E1-F1 已验证；R3-S1-R104-E1-F2 已验证；链接 可打开（200，标题「Research」）
 S1-R104-E2 规则：无规则；链接 可打开（200，标题「Advertising case studies」）
 S1-R104-E3 R3-S1-R104-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 5 个、sitemap 同结构 21 个全部匹配
 S1-R104-E3 规则：R3-S1-R104-E3-F1 已验证；链接 可打开（200，标题「News &amp; opinion」）</t>
@@ -4915,7 +5075,7 @@
       </c>
       <c r="H104" s="3" t="inlineStr">
         <is>
-          <t>S1-R104-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 174；前缀 /research/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+          <t>S1-R104-E1: 完整：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 174；前缀 /research/ 下家族 2 个、成员 47；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=0、F2=0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R104-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 176；前缀 /case-studies/ 下家族 0 个、成员 0；前缀外同站链接 1、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -4953,7 +5113,7 @@
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>S1-R105-E1 规则：R3-S1-R105-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「NRF Membership | NRF」）
+          <t>S1-R105-E1 规则：R3-S1-R105-E1-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「NRF Membership | NRF」）
 S1-R105-E2 规则：R3-S1-R105-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「About the National Retail Federation | NRF」）</t>
         </is>
       </c>
@@ -5017,35 +5177,41 @@
       </c>
       <c r="B108" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.wppmedia\.com/news/[a-zA-Z0-9'\+\.:_£åæçéøı’-]+$</t>
+          <t>^https://www\.wppmedia\.com/thought\-leadership/research\-business\-intelligence/[a-zA-Z0-9-]+$
+^https://www\.wppmedia\.com/news/[a-zA-Z0-9'\+\.:_£åæçéøı’-]+$
+^https://www\.wppmedia\.com/thought\-leadership/this\-year\-next\-year/[a-zA-Z0-9-]+$</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
         <is>
           <t>S1-R108-E1: https://www.wppmedia.com/thought-leadership/research-business-intelligence
-  其余 9 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R108-E1.txt
+  其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R108-E1.txt
 S1-R108-E2: https://www.wppmedia.com/news
   其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R108-E2.txt
 S1-R108-E3: https://www.wppmedia.com/thought-leadership/this-year-next-year
-  其余 5 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R108-E3.txt</t>
+  其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R108-E3.txt</t>
         </is>
       </c>
       <c r="D108" s="3" t="inlineStr">
         <is>
-          <t>S1-R108-E2 R3-S1-R108-E2-F1: https://www.wppmedia.com/news/ai-powered-intelligence；https://www.wppmedia.com/news/comvergence-h1-2026（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R108-E1 R3-S1-R108-E1-F1: https://www.wppmedia.com/thought-leadership/research-business-intelligence/how-humans-decide-understanding-receptivity；https://www.wppmedia.com/thought-leadership/research-business-intelligence/How-Humans-Decide-primed-for-preference（已落地核验 200，公开访问，2026-10-26）
+S1-R108-E2 R3-S1-R108-E2-F1: https://www.wppmedia.com/news/ai-powered-intelligence；https://www.wppmedia.com/news/comvergence-h1-2026（已落地核验 200，公开访问，2026-10-26）
+S1-R108-E3 R3-S1-R108-E3-F1: https://www.wppmedia.com/thought-leadership/this-year-next-year/midyear-2026；https://www.wppmedia.com/thought-leadership/this-year-next-year/December-2025（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
         <is>
-          <t>S1-R108-E1 规则：R3-S1-R108-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「WPP Media | Research &amp; Business Intelligence」）
+          <t>S1-R108-E1 R3-S1-R108-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN5；覆盖检查：列表 7 个、sitemap 同结构 7 个全部匹配
+S1-R108-E1 规则：R3-S1-R108-E1-F1 已验证；链接 可打开（200，标题「WPP Media | Research &amp; Business Intelligence」）
 S1-R108-E2 R3-S1-R108-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 12 个、sitemap 同结构 497 个全部匹配
 S1-R108-E2 规则：R3-S1-R108-E2-F1 已验证；链接 可打开（200，标题「WPP Media News | Insights, and Industry Impact」）
-S1-R108-E3 规则：R3-S1-R108-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「This Year Next Year | WPP Media」）</t>
+S1-R108-E3 R3-S1-R108-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN5；覆盖检查：列表 4 个、sitemap 同结构 3 个全部匹配
+S1-R108-E3 规则：R3-S1-R108-E3-F1 已验证；链接 可打开（200，标题「This Year Next Year | WPP Media」）</t>
         </is>
       </c>
       <c r="G108" s="3" t="inlineStr">
@@ -5138,22 +5304,31 @@
           <t>https://www.ogilvy.com/cn/ideas</t>
         </is>
       </c>
-      <c r="B111" s="4" t="inlineStr"/>
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.ogilvy\.com/cn/ideas/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
           <t>S1-R111-E1: https://www.ogilvy.com/cn/ideas
-  其余 104 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R111-E1.txt</t>
-        </is>
-      </c>
-      <c r="D111" s="3" t="inlineStr"/>
+  其余 3 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R111-E1.txt</t>
+        </is>
+      </c>
+      <c r="D111" s="3" t="inlineStr">
+        <is>
+          <t>S1-R111-E1 R3-S1-R111-E1-F1: https://www.ogilvy.com/cn/ideas/aomeironghuo-2024-dazhonghuaquaifeijiangzuijushixiaodailigongsiwangluo；https://www.ogilvy.com/cn/ideas/aomeiyatai-2024-zengzhangzhishudongchashichangqushiyinlingpinpaijiesuozengzhangxinlujing（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E111" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>S1-R111-E1 规则：R3-S1-R111-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Ideas | Ogilvy China」）</t>
+          <t>S1-R111-E1 R3-S1-R111-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN4；覆盖检查：列表 101 个、sitemap 同结构 0 个全部匹配
+S1-R111-E1 规则：R3-S1-R111-E1-F1 已验证；链接 可打开（200，标题「Ideas | Ogilvy China」）</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -5269,7 +5444,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>S1-R114-E1 规则：R3-S1-R114-E1-F1 部分验证（候选）（归纳样本跳到其他页面 1）；链接 可打开（200，标题「Resources &amp; Guides | Amplitude」）
+          <t>S1-R114-E1 规则：R3-S1-R114-E1-F1 部分验证（候选）（归纳样本跳到家族外页面 1：https://amplitude.com/resources/forrester-wave-report → https://amplitude.com/blog/roi-of-amplitude）；链接 可打开（200，标题「Resources &amp; Guides | Amplitude」）
 S1-R114-E2 R3-S1-R114-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 16 个、sitemap 同结构 1504 个全部匹配
 S1-R114-E2 R3-S1-R114-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 5 个、sitemap 同结构 580 个全部匹配
 S1-R114-E2 规则：R3-S1-R114-E2-F1 已验证；R3-S1-R114-E2-F2 已验证；链接 可打开（200，标题「Amplitude Blog - Product Best Practices &amp; More」）</t>
@@ -5303,18 +5478,20 @@
       </c>
       <c r="B115" s="4" t="inlineStr">
         <is>
-          <t>^https://analyticpartners\.com/knowledge\-hub/resources/[a-z0-9-]+/$</t>
+          <t>^https://analyticpartners\.com/knowledge\-hub/[a-z-]+/$
+^https://analyticpartners\.com/knowledge\-hub/resources/[a-z0-9-]+/$</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
         <is>
           <t>S1-R115-E1: https://analyticpartners.com/knowledge-hub/
-  其余 26 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R115-E1.txt</t>
+  其余 21 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R115-E1.txt</t>
         </is>
       </c>
       <c r="D115" s="3" t="inlineStr">
         <is>
-          <t>S1-R115-E1 R3-S1-R115-E1-F2: https://analyticpartners.com/knowledge-hub/resources/empower-your-analytics-how-leaders-operationalize-decisioning-and-generate-millions-in-returns/；https://analyticpartners.com/knowledge-hub/resources/cfo-and-cmo-strategy-guide-a-collaboration-to-drive-growth/（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R115-E1 R3-S1-R115-E1-F1: https://analyticpartners.com/knowledge-hub/blog/；https://analyticpartners.com/knowledge-hub/customer-stories/（已落地核验 200，公开访问，2026-10-26）
+S1-R115-E1 R3-S1-R115-E1-F2: https://analyticpartners.com/knowledge-hub/resources/empower-your-analytics-how-leaders-operationalize-decisioning-and-generate-millions-in-returns/；https://analyticpartners.com/knowledge-hub/resources/cfo-and-cmo-strategy-guide-a-collaboration-to-drive-growth/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E115" s="3" t="inlineStr">
@@ -5324,8 +5501,9 @@
       </c>
       <c r="F115" s="3" t="inlineStr">
         <is>
-          <t>S1-R115-E1 R3-S1-R115-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 4 个、sitemap 同结构 48 个全部匹配
-S1-R115-E1 规则：R3-S1-R115-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R115-E1-F2 已验证；链接 可打开（200，标题「Knowledge Hub | Analytic Partners」）</t>
+          <t>S1-R115-E1 R3-S1-R115-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 5 个、sitemap 同结构 5 个全部匹配
+S1-R115-E1 R3-S1-R115-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 4 个、sitemap 同结构 48 个全部匹配
+S1-R115-E1 规则：R3-S1-R115-E1-F1 已验证；R3-S1-R115-E1-F2 已验证；链接 可打开（200，标题「Knowledge Hub | Analytic Partners」）</t>
         </is>
       </c>
       <c r="G115" s="3" t="inlineStr">
@@ -5354,7 +5532,8 @@
       </c>
       <c r="B116" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.appsflyer\.com/resources/reports/[a-z0-9-]+/$</t>
+          <t>^https://www\.appsflyer\.com/resources/reports/[a-z0-9-]+/$
+^https://www\.appsflyer\.com/blog/[a-z-]+/[a-z0-9_-]+/$</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -5362,24 +5541,26 @@
           <t>S1-R116-E1: https://www.appsflyer.com/resources/
   其余 35 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R116-E1.txt
 S1-R116-E2: https://www.appsflyer.com/blog/
-  其余 56 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R116-E2.txt</t>
+  其余 35 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R116-E2.txt</t>
         </is>
       </c>
       <c r="D116" s="3" t="inlineStr">
         <is>
-          <t>S1-R116-E1 R3-S1-R116-E1-F1: https://www.appsflyer.com/resources/reports/africa-marketing-2024-report/；https://www.appsflyer.com/resources/reports/creative-optimization/（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R116-E1 R3-S1-R116-E1-F1: https://www.appsflyer.com/resources/reports/africa-marketing-2024-report/；https://www.appsflyer.com/resources/reports/creative-optimization/（已落地核验 200，公开访问，2026-10-26）
+S1-R116-E2 R3-S1-R116-E2-F1: https://www.appsflyer.com/blog/industries/entertainment/；https://www.appsflyer.com/blog/deep-linking/facebook-deep-link/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E116" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F116" s="3" t="inlineStr">
         <is>
           <t>S1-R116-E1 R3-S1-R116-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 13 个、sitemap 同结构 65 个全部匹配
 S1-R116-E1 规则：R3-S1-R116-E1-F1 已验证；链接 可打开（200，标题「Report Lobby - AppsFlyer」）
-S1-R116-E2 规则：R3-S1-R116-E2-F1 部分验证（候选）（机械门未通过：有正例未完成落地身份核验）；链接 可打开（200，标题「AppsFlyer Blog: Mobile Attribution, Cross-Platform」）</t>
+S1-R116-E2 R3-S1-R116-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP1/FP0/FN0/TN4；覆盖检查：列表 21 个、sitemap 同结构 828 个全部匹配
+S1-R116-E2 规则：R3-S1-R116-E2-F1 已验证；链接 可打开（200，标题「AppsFlyer Blog: Mobile Attribution, Cross-Platform」）</t>
         </is>
       </c>
       <c r="G116" s="3" t="inlineStr">
@@ -5392,7 +5573,7 @@
         <is>
           <t>S1-R116-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 1 个、成员 13；前缀外同站链接 35、文件 0；sitemap 中同结构但不在列表的 URL：F1=52
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R116-E2: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 21；前缀外同站链接 34、文件 0；sitemap 中同结构但不在列表的 URL：F1=807
+S1-R116-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 21；前缀外同站链接 34、文件 0；sitemap 中同结构但不在列表的 URL：F1=807
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -5426,7 +5607,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>S1-R117-E1 规则：R3-S1-R117-E1-F1 部分验证（候选）（机械门未通过：留出反例 0&lt;3；归纳样本跳到其他页面 1）；链接 可打开（200，标题「Mobile Growth Resources and Research | Branch」）
+          <t>S1-R117-E1 规则：R3-S1-R117-E1-F1 部分验证（候选）（归纳样本跳到家族外页面 1：https://www.branch.io/resources/news/branch-expands-ai-measurement-with-chatgpt-ads-attribution-across-app-web-and-desktop/ → https://www.prnewswire.com/news-releases/branch-expands-ai-measurement-with-chatgpt-ads-attribution-across-app-web-and-desktop-302888520.html）；链接 可打开（200，标题「Mobile Growth Resources and Research | Branch」）
 S1-R117-E2 规则：无规则；链接 可打开（200，标题「How Branch Helps Drive Mobile Growth - Use Cases |」）</t>
         </is>
       </c>
@@ -5465,6 +5646,7 @@
         <is>
           <t>^https://www\.brandwatch\.com/blog/[a-z0-9-]+/$
 ^https://www\.brandwatch\.com/blog/[a-z]+/[a-z0-9-]+/$
+^https://www\.brandwatch\.com/social\-media\-glossary/[a-z-]+/$
 ^https://www\.brandwatch\.com/case\-studies/[a-z0-9-]+/$</t>
         </is>
       </c>
@@ -5477,7 +5659,7 @@
 S1-R118-E3: https://www.brandwatch.com/guides/
   其余 104 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R118-E3.txt
 S1-R118-E4: https://www.brandwatch.com/social-media-glossary/
-  其余 116 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R118-E4.txt
+  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R118-E4.txt
 S1-R118-E6: https://www.brandwatch.com/case-studies/
   其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R118-E6.txt</t>
         </is>
@@ -5486,12 +5668,13 @@
         <is>
           <t>S1-R118-E2 R3-S1-R118-E2-F1: https://www.brandwatch.com/blog/customer-story-co-ops-support-of-the-reverseadvent-campaign/；https://www.brandwatch.com/blog/brandwatch-named-leader-idc-marketscape-social-marketing-software-large-enterprises/（已落地核验 200，公开访问，2026-10-26）
 S1-R118-E2 R3-S1-R118-E2-F2: https://www.brandwatch.com/blog/author/aj-wilcox/；https://www.brandwatch.com/blog/author/adam-speight/（已落地核验 200，公开访问，2026-10-26）
+S1-R118-E4 R3-S1-R118-E4-F1: https://www.brandwatch.com/social-media-glossary/content-pillars/；https://www.brandwatch.com/social-media-glossary/carousel/（已落地核验 200，公开访问，2026-10-26）
 S1-R118-E6 R3-S1-R118-E6-F1: https://www.brandwatch.com/case-studies/barilla-it/；https://www.brandwatch.com/case-studies/art-of-the-possible/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E118" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 链接保留；E4 链接保留；E6 正则+链接保留；E5 host免提</t>
+          <t>E1 链接保留；E2 正则+链接保留；E3 链接保留；E4 正则+链接保留；E6 正则+链接保留；E5 host免提</t>
         </is>
       </c>
       <c r="F118" s="3" t="inlineStr">
@@ -5501,7 +5684,8 @@
 S1-R118-E2 R3-S1-R118-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 11 个、sitemap 同结构 423 个全部匹配
 S1-R118-E2 规则：R3-S1-R118-E2-F1 已验证；R3-S1-R118-E2-F2 已验证；链接 可打开（200，标题「Blog |  Brandwatch」）
 S1-R118-E3 规则：无规则；链接 可打开（200，标题「Consumer and Social Media Marketing Guides | Brand」）
-S1-R118-E4 规则：R3-S1-R118-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Social Media Glossary &amp; Marketing Terms | Brandwat」）
+S1-R118-E4 R3-S1-R118-E4-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN5；覆盖检查：列表 110 个、sitemap 同结构 110 个全部匹配
+S1-R118-E4 规则：R3-S1-R118-E4-F1 已验证；链接 可打开（200，标题「Social Media Glossary &amp; Marketing Terms | Brandwat」）
 S1-R118-E6 R3-S1-R118-E6-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 76 个、sitemap 同结构 85 个全部匹配
 S1-R118-E6 规则：R3-S1-R118-E6-F1 已验证；链接 可打开（200，标题「Brandwatch Case Studies | Real Client Results」）</t>
         </is>
@@ -5737,20 +5921,22 @@
       </c>
       <c r="B122" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.hootsuite\.com/resources/[a-z-]+/[a-z0-9-]+$</t>
+          <t>^https://www\.hootsuite\.com/resources/[a-z-]+/[a-z0-9-]+$
+^https://www\.hootsuite\.com/resources/[a-z0-9-]+$</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
         <is>
           <t>S1-R122-E1: https://www.hootsuite.com/resources/
-  其余 11 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R122-E1.txt
+  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R122-E1.txt
 S1-R122-E3: https://blog.hootsuite.com/resources/
   其余 877 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R122-E3.txt</t>
         </is>
       </c>
       <c r="D122" s="3" t="inlineStr">
         <is>
-          <t>S1-R122-E1 R3-S1-R122-E1-F1: https://www.hootsuite.com/resources/blog/healthcare-social-media-policy-template；https://www.hootsuite.com/resources/blog/competitive-analysis-template（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R122-E1 R3-S1-R122-E1-F1: https://www.hootsuite.com/resources/blog/healthcare-social-media-policy-template；https://www.hootsuite.com/resources/blog/competitive-analysis-template（已落地核验 200，公开访问，2026-10-26）
+S1-R122-E1 R3-S1-R122-E1-F2: https://www.hootsuite.com/resources/croda；https://www.hootsuite.com/resources/influencer-marketing-myths（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E122" s="3" t="inlineStr">
@@ -5761,7 +5947,8 @@
       <c r="F122" s="3" t="inlineStr">
         <is>
           <t>S1-R122-E1 R3-S1-R122-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 6 个、sitemap 同结构 126 个全部匹配
-S1-R122-E1 规则：R3-S1-R122-E1-F1 已验证；R3-S1-R122-E1-F2 部分验证（候选）（归纳样本跳到其他页面 1）；链接 可打开（200，标题「Social Media Resources: Templates, Case Studies, R」）
+S1-R122-E1 R3-S1-R122-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP5/FP0/FN0/TN6；覆盖检查：列表 5 个、sitemap 同结构 143 个全部匹配
+S1-R122-E1 规则：R3-S1-R122-E1-F1 已验证；R3-S1-R122-E1-F2 已验证；链接 可打开（200，标题「Social Media Resources: Templates, Case Studies, R」）
 S1-R122-E3 规则：无规则；链接 可打开（200，标题「Free Social Media Resources, Tools and Templates |」）</t>
         </is>
       </c>
@@ -5773,7 +5960,7 @@
       </c>
       <c r="H122" s="3" t="inlineStr">
         <is>
-          <t>S1-R122-E1: 部分：静态请求 3 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 2 个、成员 11；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=121、F2=139
+          <t>S1-R122-E1: 完整（列表+sitemap 合并枚举）：静态请求 3 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 2 个、成员 11；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=121、F2=139
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R122-E3: 完整（枚举结束，无独立全集对账）：静态请求 71 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 155；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 877、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -5795,33 +5982,48 @@
 https://www.hubspot.com/resources</t>
         </is>
       </c>
-      <c r="B123" s="4" t="inlineStr"/>
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>^https://blog\.hubspot\.com/marketing/[a-z0-9_-]+$
+^https://blog\.hubspot\.com/sales/[a-zA-Z0-9%ü-]+$
+^https://blog\.hubspot\.com/service/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C123" s="3" t="inlineStr">
         <is>
           <t>S1-R123-E1: https://blog.hubspot.com/marketing
-  其余 3888 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E1.txt
+  其余 391 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E1.txt
 S1-R123-E2: https://blog.hubspot.com/sales
-  其余 1606 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E2.txt
+  其余 8 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E2.txt
 S1-R123-E3: https://blog.hubspot.com/service
-  其余 781 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E3.txt
+  其余 7 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E3.txt
 S1-R123-E4: https://blog.hubspot.com/website
   其余 1347 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E4.txt
 S1-R123-E5: https://www.hubspot.com/resources
   其余 56 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E5.txt</t>
         </is>
       </c>
-      <c r="D123" s="3" t="inlineStr"/>
+      <c r="D123" s="3" t="inlineStr">
+        <is>
+          <t>S1-R123-E1 R3-S1-R123-E1-F1: https://blog.hubspot.com/marketing/ai-search-presence；https://blog.hubspot.com/marketing/gain-instagram-followers（已落地核验 200，公开访问，2026-10-26）
+S1-R123-E2 R3-S1-R123-E2-F1: https://blog.hubspot.com/sales/ai-franchise；https://blog.hubspot.com/sales/avoid-burnout-q4（已落地核验 200，公开访问，2026-10-26）
+S1-R123-E3 R3-S1-R123-E3-F1: https://blog.hubspot.com/service/apology-letter-to-customers；https://blog.hubspot.com/service/customer-success-metrics（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留；E3 链接保留；E4 链接保留；E5 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 链接保留；E5 链接保留</t>
         </is>
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>S1-R123-E1 规则：R3-S1-R123-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R123-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R123-E1-F3 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The HubSpot Marketing Blog」）
-S1-R123-E2 规则：R3-S1-R123-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The HubSpot Sales Blog」）
-S1-R123-E3 规则：R3-S1-R123-E3-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The HubSpot Customer Service Blog」）
-S1-R123-E4 规则：R3-S1-R123-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）；归纳样本跳到其他页面 2）；链接 可打开（200，标题「The HubSpot Website Blog」）
+          <t>S1-R123-E1 R3-S1-R123-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(later_pagination_pages) TP6/FP0/FN0/TN6；覆盖检查：列表 3497 个、sitemap 同结构 3497 个全部匹配
+S1-R123-E1 规则：R3-S1-R123-E1-F1 已验证；R3-S1-R123-E1-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R123-E1-F3 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The HubSpot Marketing Blog」）
+S1-R123-E2 R3-S1-R123-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 1598 个、sitemap 同结构 1597 个全部匹配
+S1-R123-E2 规则：R3-S1-R123-E2-F1 已验证；链接 可打开（200，标题「The HubSpot Sales Blog」）
+S1-R123-E3 R3-S1-R123-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(later_pagination_pages) TP6/FP0/FN0/TN4；覆盖检查：列表 774 个、sitemap 同结构 774 个全部匹配
+S1-R123-E3 规则：R3-S1-R123-E3-F1 已验证；链接 可打开（200，标题「The HubSpot Customer Service Blog」）
+S1-R123-E4 规则：R3-S1-R123-E4-F1 部分验证（候选）（归纳样本跳到家族外页面 2：https://blog.hubspot.com/website/html-elements → https://blog.hubspot.com/website；https://blog.hubspot.com/website/html-span → https://blog.hubspot.com/website）；链接 可打开（200，标题「The HubSpot Website Blog」）
 S1-R123-E5 规则：无规则；链接 可打开（200，标题「Free Resources from HubSpot | Templates, Ebooks, &amp;」）</t>
         </is>
       </c>
@@ -5838,7 +6040,7 @@
         <is>
           <t>S1-R123-E1: 完整：静态请求 196 页（入口+分页），未完成分页 0；前缀 /marketing/ 下家族 3 个、成员 3503；前缀外同站链接 376、文件 0；sitemap 中同结构但不在列表的 URL：F1=0、F2=0、F3=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R123-E2: 部分：静态请求 81 页（入口+分页），未完成分页 0；前缀 /sales/ 下家族 1 个、成员 1598；前缀外同站链接 5、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
+S1-R123-E2: 完整（列表+sitemap 合并枚举）：静态请求 81 页（入口+分页），未完成分页 0；前缀 /sales/ 下家族 1 个、成员 1598；前缀外同站链接 5、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R123-E3: 完整：静态请求 40 页（入口+分页），未完成分页 0；前缀 /service/ 下家族 1 个、成员 774；前缀外同站链接 4、文件 0；sitemap 中同结构但不在列表的 URL：F1=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -5860,22 +6062,31 @@
           <t>https://www.intercom.com/blog/</t>
         </is>
       </c>
-      <c r="B124" s="4" t="inlineStr"/>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.intercom\.com/blog/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
           <t>S1-R124-E1: https://www.intercom.com/blog/
-  其余 1274 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R124-E1.txt</t>
-        </is>
-      </c>
-      <c r="D124" s="3" t="inlineStr"/>
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R124-E1.txt</t>
+        </is>
+      </c>
+      <c r="D124" s="3" t="inlineStr">
+        <is>
+          <t>S1-R124-E1 R3-S1-R124-E1-F1: https://www.intercom.com/blog/podcasts；https://www.intercom.com/blog/5-new-intercom-messenger-apps（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E124" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>S1-R124-E1 规则：无规则；链接 可打开（200，标题「Blog | Intercom」）</t>
+          <t>S1-R124-E1 R3-S1-R124-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP2/FP0/FN0/TN5；覆盖检查：列表 1274 个、sitemap 同结构 1229 个全部匹配
+S1-R124-E1 规则：R3-S1-R124-E1-F1 已验证；链接 可打开（200，标题「Blog | Intercom」）</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -5885,14 +6096,13 @@
       </c>
       <c r="H124" s="3" t="inlineStr">
         <is>
-          <t>S1-R124-E1: 完整：静态请求 64 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 1274；前缀外同站链接 0、文件 0
+          <t>S1-R124-E1: 完整（列表+sitemap 合并枚举）：静态请求 64 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 1274；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=2
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>行边界为重建：内联粘贴丢失引号，按连续同注册域分组得 152 行（107 个 URL 单元格+45 个“/”行），与前轮检查点计数一致，待与原始文件核对
-S1-R124-E1 R3-S1-R124-E1-F1 未成规则：归纳样本落地不足 3 个正常页面</t>
+          <t>行边界为重建：内联粘贴丢失引号，按连续同注册域分组得 152 行（107 个 URL 单元格+45 个“/”行），与前轮检查点计数一致，待与原始文件核对</t>
         </is>
       </c>
     </row>
@@ -6070,13 +6280,14 @@
       <c r="B128" s="4" t="inlineStr">
         <is>
           <t>^https://www\.meltwater\.com/en/blog/[a-z0-9_-]+$
+^https://www\.meltwater\.com/en/blog/[a-z]+/[a-z-]+$
 ^https://www\.meltwater\.com/en/resources/[a-z0-9_-]+$</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
           <t>S1-R128-E1: https://www.meltwater.com/en/blog
-  其余 21 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R128-E1.txt
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R128-E1.txt
 S1-R128-E2: https://www.meltwater.com/en/resources
   其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R128-E2.txt</t>
         </is>
@@ -6084,6 +6295,7 @@
       <c r="D128" s="3" t="inlineStr">
         <is>
           <t>S1-R128-E1 R3-S1-R128-E1-F1: https://www.meltwater.com/en/blog/3-steps-to-social-media-holiday-strategy-with-examples；https://www.meltwater.com/en/blog/beyond-polarity-attitude-analysis（已落地核验 200，公开访问，2026-10-26）
+S1-R128-E1 R3-S1-R128-E1-F2: https://www.meltwater.com/en/blog/category/brand-management；https://www.meltwater.com/en/blog/category/customer-journey（已落地核验 200，公开访问，2026-10-26）
 S1-R128-E2 R3-S1-R128-E2-F1: https://www.meltwater.com/en/resources/2024-consumer-insights-food-beverage；https://www.meltwater.com/en/resources/ai-visibility-australian-higher-education（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
@@ -6095,7 +6307,8 @@
       <c r="F128" s="3" t="inlineStr">
         <is>
           <t>S1-R128-E1 R3-S1-R128-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 36 个、sitemap 同结构 1313 个全部匹配
-S1-R128-E1 规则：R3-S1-R128-E1-F1 已验证；R3-S1-R128-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「The Meltwater Blog」）
+S1-R128-E1 R3-S1-R128-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP5/FP0/FN0/TN7；覆盖检查：列表 21 个、sitemap 同结构 21 个全部匹配
+S1-R128-E1 规则：R3-S1-R128-E1-F1 已验证；R3-S1-R128-E1-F2 已验证；链接 可打开（200，标题「The Meltwater Blog」）
 S1-R128-E2 R3-S1-R128-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 27 个、sitemap 同结构 473 个全部匹配
 S1-R128-E2 规则：R3-S1-R128-E2-F1 已验证；链接 可打开（200，标题「Browse our library of ebooks, webinars and videos」）</t>
         </is>
@@ -6210,7 +6423,7 @@
 S1-R130-E2: https://www.qualtrics.com/news/
   其余 5 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R130-E2.txt
 S1-R130-E3: https://www.qualtrics.com/resources/
-  其余 240 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R130-E3.txt
+  其余 242 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R130-E3.txt
 S1-R130-E4: https://www.qualtrics.com/customers/
   其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R130-E4.txt</t>
         </is>
@@ -6252,7 +6465,7 @@
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R130-E2: 完整（列表+sitemap 合并枚举）：静态请求 32 页（入口+分页），未完成分页 0；前缀 /news/ 下家族 1 个、成员 363；前缀外同站链接 3、文件 1；sitemap 中同结构但不在列表的 URL：F1=4
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R130-E3: 完整（枚举结束，无独立全集对账）：静态请求 21 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 292；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 240、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+S1-R130-E3: 完整（枚举结束，无独立全集对账）：静态请求 21 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 292；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 240、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R130-E4: 完整（列表+sitemap 合并枚举）：静态请求 7 页（入口+分页），未完成分页 0；前缀 /customers/ 下家族 1 个、成员 62；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=2
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -6310,7 +6523,7 @@
       </c>
       <c r="H131" s="3" t="inlineStr">
         <is>
-          <t>S1-R131-E1: 部分：静态请求 486 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 3 个、成员 2335；前缀外同站链接 430、文件 0；sitemap 中同结构但不在列表的 URL：F1=80、F2=1、F3=0
+          <t>S1-R131-E1: 完整（列表+sitemap 合并枚举）：静态请求 486 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 3 个、成员 2335；前缀外同站链接 430、文件 0；sitemap 中同结构但不在列表的 URL：F1=80、F2=1、F3=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -6328,18 +6541,20 @@
       </c>
       <c r="B132" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.shopify\.com/blog/[a-z0-9-]+$</t>
+          <t>^https://www\.shopify\.com/blog/[a-z0-9-]+$
+^https://www\.shopify\.com/blog/[a-z]+/[a-zA-Z0-9%-]+$</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
           <t>S1-R132-E1: https://www.shopify.com/blog/
-  其余 18 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R132-E1.txt</t>
+  其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R132-E1.txt</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>S1-R132-E1 R3-S1-R132-E1-F1: https://www.shopify.com/blog/email-marketing；https://www.shopify.com/blog/b2b-marketing-kpis（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R132-E1 R3-S1-R132-E1-F1: https://www.shopify.com/blog/best-web-hosting-services；https://www.shopify.com/blog/b2b-marketing-kpis（已落地核验 200，公开访问，2026-10-26）
+S1-R132-E1 R3-S1-R132-E1-F2: https://www.shopify.com/blog/authors/altaira-northe；https://www.shopify.com/blog/authors/shuang-esther-shan（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
@@ -6349,8 +6564,9 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>S1-R132-E1 R3-S1-R132-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP3/FP0/FN0/TN7；覆盖检查：列表 36 个、sitemap 同结构 5 个全部匹配
-S1-R132-E1 规则：R3-S1-R132-E1-F1 已验证；R3-S1-R132-E1-F2 部分验证（候选）（机械门未通过：有正例未完成落地身份核验；归纳样本跳到其他页面 1）；链接 可打开（200，标题「Ecommerce Marketing Blog - Ecommerce News, Online 」）</t>
+          <t>S1-R132-E1 R3-S1-R132-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 36 个、sitemap 同结构 6566 个全部匹配
+S1-R132-E1 R3-S1-R132-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP3/FP0/FN0/TN6；覆盖检查：列表 16 个、sitemap 同结构 326 个全部匹配
+S1-R132-E1 规则：R3-S1-R132-E1-F1 已验证；R3-S1-R132-E1-F2 已验证；链接 可打开（200，标题「Ecommerce Marketing Blog - Ecommerce News, Online 」）</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -6360,7 +6576,7 @@
       </c>
       <c r="H132" s="3" t="inlineStr">
         <is>
-          <t>S1-R132-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 52；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=3、F2=323
+          <t>S1-R132-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 52；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=6530、F2=323
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -6434,18 +6650,20 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.sistrix\.com/blog/[a-z0-9%_-]+/?$</t>
+          <t>^https://www\.sistrix\.com/blog/[a-z0-9%_-]+/?$
+^https://www\.sistrix\.com/blog/archive/\?selected=[0-9]*$</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
           <t>S1-R135-E1: https://www.sistrix.com/blog/
-  其余 44 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R135-E1.txt</t>
+  其余 24 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R135-E1.txt</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
         <is>
-          <t>S1-R135-E1 R3-S1-R135-E1-F1: https://www.sistrix.com/blog/ancillary-copyright-law-how-much-journalistic-content-is-found-in-google-search/；https://www.sistrix.com/blog/core-web-vitals-wix-vs-wordpress-shopify-vs-shopware-whats-fastest/（已落地核验 200，公开访问，2026-10-26）</t>
+          <t>S1-R135-E1 R3-S1-R135-E1-F1: https://www.sistrix.com/blog/ancillary-copyright-law-how-much-journalistic-content-is-found-in-google-search/；https://www.sistrix.com/blog/core-web-vitals-wix-vs-wordpress-shopify-vs-shopware-whats-fastest/（已落地核验 200，公开访问，2026-10-26）
+S1-R135-E1 R3-S1-R135-E1-F2: https://www.sistrix.com/blog/archive/?selected=2008；https://www.sistrix.com/blog/archive/?selected=2007（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E135" s="3" t="inlineStr">
@@ -6456,7 +6674,8 @@
       <c r="F135" s="3" t="inlineStr">
         <is>
           <t>S1-R135-E1 R3-S1-R135-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 25 个、sitemap 同结构 840 个全部匹配
-S1-R135-E1 规则：R3-S1-R135-E1-F1 已验证；R3-S1-R135-E1-F2 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「SISTRIX SEO Blog, studies and expert content - SIS」）</t>
+S1-R135-E1 R3-S1-R135-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP5/FP0/FN0/TN7；覆盖检查：列表 20 个、sitemap 同结构 0 个全部匹配
+S1-R135-E1 规则：R3-S1-R135-E1-F1 已验证；R3-S1-R135-E1-F2 已验证；链接 可打开（200，标题「SISTRIX SEO Blog, studies and expert content - SIS」）</t>
         </is>
       </c>
       <c r="G135" s="3" t="inlineStr">
@@ -6544,9 +6763,9 @@
           <t>S1-R137-E1: https://www.talkwalker.com/blog
   其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R137-E1.txt
 S1-R137-E2: https://www.talkwalker.com/resources?category=Reports
-  其余 34 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R137-E2.txt
+  其余 35 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R137-E2.txt
 S1-R137-E3: https://www.talkwalker.com/resources
-  其余 24 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R137-E3.txt</t>
+  其余 25 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R137-E3.txt</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
@@ -6578,9 +6797,9 @@
         <is>
           <t>S1-R137-E1: 完整（列表+sitemap 合并枚举）：静态请求 3 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 15；前缀外同站链接 13、文件 0；sitemap 中同结构但不在列表的 URL：F1=165
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R137-E2: 完整（枚举结束，无独立全集对账）：静态请求 10 页（入口+分页），未完成分页 0；浏览器渲染 3 轮、点击加载更多 0 次、渲染后链接 105；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 34、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R137-E3: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 110；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 24、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
+S1-R137-E2: 完整（枚举结束，无独立全集对账）：静态请求 10 页（入口+分页），未完成分页 0；浏览器渲染 3 轮、点击加载更多 0 次、渲染后链接 105；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 34、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R137-E3: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 110；前缀 /resources/ 下家族 0 个、成员 0；前缀外同站链接 24、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -6622,7 +6841,7 @@
       </c>
       <c r="F138" s="3" t="inlineStr">
         <is>
-          <t>S1-R138-E1 规则：R3-S1-R138-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Landing page optimization resources | Unbounce blo」）
+          <t>S1-R138-E1 规则：R3-S1-R138-E1-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Landing page optimization resources | Unbounce blo」）
 S1-R138-E2 R3-S1-R138-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP1/FP0/FN0/TN5；覆盖检查：列表 9 个、sitemap 同结构 0 个全部匹配
 S1-R138-E2 规则：R3-S1-R138-E2-F1 已验证；链接 可打开（200，标题「Average conversion rate by industry benchmark repo」）</t>
         </is>
@@ -6679,7 +6898,7 @@
       </c>
       <c r="F139" s="3" t="inlineStr">
         <is>
-          <t>S1-R139-E1 R3-S1-R139-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 2597 个、sitemap 同结构 2680 个全部匹配
+          <t>S1-R139-E1 R3-S1-R139-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 2597 个、sitemap 同结构 2685 个全部匹配
 S1-R139-E1 规则：R3-S1-R139-E1-F1 已验证；链接 可打开（200，标题「Blog - We Are Social UK」）
 S1-R139-E2 规则：无规则；链接 可打开（200，标题「Our Reports - We Are Social UK」）</t>
         </is>
@@ -6692,7 +6911,7 @@
       </c>
       <c r="H139" s="3" t="inlineStr">
         <is>
-          <t>S1-R139-E1: 部分：静态请求 269 页（入口+分页），未完成分页 0；前缀 /uk/blog/ 下家族 1 个、成员 2597；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=90
+          <t>S1-R139-E1: 完整（列表+sitemap 合并枚举）：静态请求 269 页（入口+分页），未完成分页 0；前缀 /uk/blog/ 下家族 1 个、成员 2597；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=91
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R139-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /uk/reports/ 下家族 0 个、成员 0；前缀外同站链接 12、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -6716,6 +6935,7 @@
       <c r="B140" s="4" t="inlineStr">
         <is>
           <t>^https://wingify\.com/blog/[a-z0-9-]+/$
+^https://wingify\.com/ebooks/[a-z0-9-]+/$
 ^https://wingify\.com/success\-stories/[a-z-]+/$</t>
         </is>
       </c>
@@ -6724,7 +6944,7 @@
           <t>S1-R140-E1: https://wingify.com/blog/
   其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R140-E1.txt
 S1-R140-E2: https://wingify.com/ebooks/
-  其余 25 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R140-E2.txt
+  其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R140-E2.txt
 S1-R140-E3: https://wingify.com/success-stories/
   其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R140-E3.txt
 S1-R140-E4: https://wingify.com/resources/
@@ -6734,19 +6954,21 @@
       <c r="D140" s="3" t="inlineStr">
         <is>
           <t>S1-R140-E1 R3-S1-R140-E1-F1: https://wingify.com/blog/feature-flags-agile-software-development/；https://wingify.com/blog/insights-into-action-wingz-ai/（已落地核验 200，公开访问，2026-10-26）
+S1-R140-E2 R3-S1-R140-E2-F1: https://wingify.com/ebooks/30-black-friday-tests-how-to-win-big-during-the-e-commerce-holiday-season/；https://wingify.com/ebooks/airline-mobile-booking-benchmark-report/（已落地核验 200，公开访问，2026-10-26）
 S1-R140-E3 R3-S1-R140-E3-F1: https://wingify.com/success-stories/defacto/；https://wingify.com/success-stories/copado/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 链接保留；E3 正则+链接保留；E4 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 链接保留</t>
         </is>
       </c>
       <c r="F140" s="3" t="inlineStr">
         <is>
           <t>S1-R140-E1 R3-S1-R140-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 12 个、sitemap 同结构 991 个全部匹配
 S1-R140-E1 规则：R3-S1-R140-E1-F1 已验证；链接 可打开（200，标题「Blog On Best Practices &amp; Insights in CRO, UX &amp; CX 」）
-S1-R140-E2 规则：R3-S1-R140-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「EBooks &amp; Guides | Wingify」）
+S1-R140-E2 R3-S1-R140-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP3/FP0/FN0/TN5；覆盖检查：列表 12 个、sitemap 同结构 0 个全部匹配
+S1-R140-E2 规则：R3-S1-R140-E2-F1 已验证；链接 可打开（200，标题「EBooks &amp; Guides | Wingify」）
 S1-R140-E3 R3-S1-R140-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP4/FP0/FN0/TN5；覆盖检查：列表 12 个、sitemap 同结构 0 个全部匹配
 S1-R140-E3 规则：R3-S1-R140-E3-F1 已验证；链接 可打开（200，标题「Customer Success Stories &amp; Case Studies | VWO」）
 S1-R140-E4 规则：无规则；链接 可打开（200，标题「Resources On Testing, Personalization, Customer Ex」）</t>
@@ -7104,7 +7326,7 @@
       <c r="B151" s="4" t="inlineStr">
         <is>
           <t>^https://www\.cbinsights\.com/research/[a-z-]+/[a-z0-9-]+/$
-^https://www\.cbinsights\.com/research/[a-z0-9-]+/$</t>
+^https://www\.cbinsights\.com/research/[a-z0-9%_-]+/$</t>
         </is>
       </c>
       <c r="C151" s="3" t="inlineStr">
@@ -7118,7 +7340,7 @@
       <c r="D151" s="3" t="inlineStr">
         <is>
           <t>S1-R151-E2 R3-S1-R151-E2-F1: https://www.cbinsights.com/research/briefing/webinar-ai-agents-driving-roi/；https://www.cbinsights.com/research/briefing/webinar-behind-the-scenes-insurtech-50-2026/（已落地核验 200，公开访问，2026-10-26）
-S1-R151-E2 R3-S1-R151-E2-F2: https://www.cbinsights.com/research/artificial-intelligence/；https://www.cbinsights.com/research/14-repeat-founders-building-agentic-commerce/（已落地核验 200，公开访问，2026-10-26）</t>
+S1-R151-E2 R3-S1-R151-E2-F2: https://www.cbinsights.com/research/asia-pacific-tech-startups-map/；https://www.cbinsights.com/research/14-repeat-founders-building-agentic-commerce/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E151" s="3" t="inlineStr">
@@ -7129,7 +7351,7 @@
       <c r="F151" s="3" t="inlineStr">
         <is>
           <t>S1-R151-E2 R3-S1-R151-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN7；覆盖检查：列表 13 个、sitemap 同结构 0 个全部匹配
-S1-R151-E2 R3-S1-R151-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP6/FP0/FN0/TN7；覆盖检查：列表 8 个、sitemap 同结构 0 个全部匹配
+S1-R151-E2 R3-S1-R151-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 8 个、sitemap 同结构 8403 个全部匹配
 S1-R151-E2 规则：R3-S1-R151-E2-F1 已验证；R3-S1-R151-E2-F2 已验证；第 2 轮：无规则；链接 可打开（200，标题「CB Insights Research」）
 S1-R151-E3 规则：无规则；第 2 轮：无规则；链接 可打开（200，标题「Strategy Terminal&lt;!-- --&gt; - CB Insights」）</t>
         </is>
@@ -7142,7 +7364,7 @@
       </c>
       <c r="H151" s="3" t="inlineStr">
         <is>
-          <t>S1-R151-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 2 个、成员 21；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=0、F2=0
+          <t>S1-R151-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 2 个、成员 21；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=0、F2=8395
   第 2 轮人工复核：部分：入口静态首轮 1 页（8100 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json
 S1-R151-E3: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 0；前缀 /strategy-terminal/ 下家族 0 个、成员 0；前缀外同站链接 45、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：部分：入口静态首轮 1 页（9994 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json</t>

</xml_diff>

<commit_message>
Apply user decision: accept listing links that land outside the family for 5 rules
4 rules become verified (Contentsquare blog, Amplitude resources, Branch
resources, HubSpot website); WIPO PATENTSCOPE stays a candidate because it
still has no independent holdout sample. 146 verified rules, 116 entries.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HW9kjaADHDgTyps9HbQ9Ce
</commit_message>
<xml_diff>
--- a/url-pattern-verification/output/round3/result-table.xlsx
+++ b/url-pattern-verification/output/round3/result-table.xlsx
@@ -1233,7 +1233,7 @@
           <t>S1-R19-E1 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP Resources」）
 S1-R19-E2 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Publications」）
 S1-R19-E3 规则：R3-S1-R19-E3-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Statistics」）
-S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本）；归纳样本跳到家族外页面 1：https://www.wipo.int/en/web/patentscope/webinar → https://www.wipo.int/en/web/patentscope/webinar/index）；R3-S1-R19-E4-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
+S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E4-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
 S1-R19-E6 R3-S1-R19-E6-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP3/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
 S1-R19-E6 规则：R3-S1-R19-E6-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E6-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Brand Database」）
 S1-R19-E8 规则：R3-S1-R19-E8-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Design Database」）
@@ -5419,32 +5419,35 @@
       </c>
       <c r="B114" s="4" t="inlineStr">
         <is>
-          <t>^https://amplitude\.com/blog/[a-zA-Z0-9-]+$
+          <t>^https://amplitude\.com/resources/[a-zA-Z0-9_-]+$
+^https://amplitude\.com/blog/[a-zA-Z0-9-]+$
 ^https://amplitude\.com/blog/[a-z]+/[a-zA-Z0-9-]+$</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
         <is>
           <t>S1-R114-E1: https://amplitude.com/resources
-  其余 19 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R114-E1.txt
+  其余 5 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R114-E1.txt
 S1-R114-E2: https://amplitude.com/blog
   其余 1 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R114-E2.txt</t>
         </is>
       </c>
       <c r="D114" s="3" t="inlineStr">
         <is>
-          <t>S1-R114-E2 R3-S1-R114-E2-F1: https://amplitude.com/blog/ai-agents-confluencevc；https://amplitude.com/blog/agent-data-security（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R114-E1 R3-S1-R114-E1-F1: https://amplitude.com/resources/digital-product-adoption-guide；https://amplitude.com/resources/north-star-playbook（已落地核验 200，公开访问，2026-10-26）
+S1-R114-E2 R3-S1-R114-E2-F1: https://amplitude.com/blog/ai-agents-confluencevc；https://amplitude.com/blog/agent-data-security（已落地核验 200，公开访问，2026-10-26）
 S1-R114-E2 R3-S1-R114-E2-F2: https://amplitude.com/blog/author/cat-perezamplitudenew-com；https://amplitude.com/blog/author/eric-kim（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E114" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 host免提</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 host免提</t>
         </is>
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>S1-R114-E1 规则：R3-S1-R114-E1-F1 部分验证（候选）（归纳样本跳到家族外页面 1：https://amplitude.com/resources/forrester-wave-report → https://amplitude.com/blog/roi-of-amplitude）；链接 可打开（200，标题「Resources &amp; Guides | Amplitude」）
+          <t>S1-R114-E1 R3-S1-R114-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 14 个、sitemap 同结构 166 个全部匹配
+S1-R114-E1 规则：R3-S1-R114-E1-F1 已验证；链接 可打开（200，标题「Resources &amp; Guides | Amplitude」）
 S1-R114-E2 R3-S1-R114-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 16 个、sitemap 同结构 1504 个全部匹配
 S1-R114-E2 R3-S1-R114-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 5 个、sitemap 同结构 580 个全部匹配
 S1-R114-E2 规则：R3-S1-R114-E2-F1 已验证；R3-S1-R114-E2-F2 已验证；链接 可打开（200，标题「Amplitude Blog - Product Best Practices &amp; More」）</t>
@@ -5458,7 +5461,7 @@
       </c>
       <c r="H114" s="3" t="inlineStr">
         <is>
-          <t>S1-R114-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 199；前缀 /resources/ 下家族 1 个、成员 14；前缀外同站链接 3、文件 2；sitemap 中同结构但不在列表的 URL：F1=152
+          <t>S1-R114-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 199；前缀 /resources/ 下家族 1 个、成员 14；前缀外同站链接 3、文件 2；sitemap 中同结构但不在列表的 URL：F1=152
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R114-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 21；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=1489、F2=575
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -5590,24 +5593,33 @@
 https://www.branch.io/use-cases/</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr"/>
+      <c r="B117" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.branch\.io/resources/[a-z-]+/[a-z0-9_-]+/$</t>
+        </is>
+      </c>
       <c r="C117" s="3" t="inlineStr">
         <is>
           <t>S1-R117-E1: https://www.branch.io/resources/
-  其余 11 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R117-E1.txt
+  其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R117-E1.txt
 S1-R117-E2: https://www.branch.io/use-cases/
   其余 29 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R117-E2.txt</t>
         </is>
       </c>
-      <c r="D117" s="3" t="inlineStr"/>
+      <c r="D117" s="3" t="inlineStr">
+        <is>
+          <t>S1-R117-E1 R3-S1-R117-E1-F1: https://www.branch.io/resources/author/rob-gioia/；https://www.branch.io/resources/blog/branch-brings-paid-and-organic-chatgpt-measurement-together/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E117" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 正则+链接保留；E2 链接保留</t>
         </is>
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>S1-R117-E1 规则：R3-S1-R117-E1-F1 部分验证（候选）（归纳样本跳到家族外页面 1：https://www.branch.io/resources/news/branch-expands-ai-measurement-with-chatgpt-ads-attribution-across-app-web-and-desktop/ → https://www.prnewswire.com/news-releases/branch-expands-ai-measurement-with-chatgpt-ads-attribution-across-app-web-and-desktop-302888520.html）；链接 可打开（200，标题「Mobile Growth Resources and Research | Branch」）
+          <t>S1-R117-E1 R3-S1-R117-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 9 个、sitemap 同结构 1329 个全部匹配
+S1-R117-E1 规则：R3-S1-R117-E1-F1 已验证；链接 可打开（200，标题「Mobile Growth Resources and Research | Branch」）
 S1-R117-E2 规则：无规则；链接 可打开（200，标题「How Branch Helps Drive Mobile Growth - Use Cases |」）</t>
         </is>
       </c>
@@ -5619,7 +5631,7 @@
       </c>
       <c r="H117" s="3" t="inlineStr">
         <is>
-          <t>S1-R117-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 1 个、成员 9；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=1321
+          <t>S1-R117-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 1 个、成员 9；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=1321
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R117-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 3 轮、点击加载更多 0 次、渲染后链接 126；前缀 /use-cases/ 下家族 0 个、成员 0；前缀外同站链接 29、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -5852,14 +5864,15 @@
       </c>
       <c r="B121" s="4" t="inlineStr">
         <is>
-          <t>^https://contentsquare\.com/ebooks\-reports/page/[0-9]+/$
+          <t>^https://contentsquare\.com/blog/[a-z0-9-]+/$
+^https://contentsquare\.com/ebooks\-reports/page/[0-9]+/$
 ^https://contentsquare\.com/guides/[a-z0-9-]+/$</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
         <is>
           <t>S1-R121-E1: https://contentsquare.com/blog/
-  其余 279 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R121-E1.txt
+  其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R121-E1.txt
 S1-R121-E2: https://contentsquare.com/ebooks-reports/
   其余 27 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R121-E2.txt
 S1-R121-E3: https://contentsquare.com/guides/
@@ -5868,18 +5881,20 @@
       </c>
       <c r="D121" s="3" t="inlineStr">
         <is>
-          <t>S1-R121-E2 R3-S1-R121-E2-F1: https://contentsquare.com/ebooks-reports/page/2/；https://contentsquare.com/ebooks-reports/page/3/（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R121-E1 R3-S1-R121-E1-F1: https://contentsquare.com/blog/behavioral-analytics-crm-data-personalization/；https://contentsquare.com/blog/how-to-track-optimize-ai-traffic/（已落地核验 200，公开访问，2026-10-26）
+S1-R121-E2 R3-S1-R121-E2-F1: https://contentsquare.com/ebooks-reports/page/2/；https://contentsquare.com/ebooks-reports/page/3/（已落地核验 200，公开访问，2026-10-26）
 S1-R121-E3 R3-S1-R121-E3-F1: https://contentsquare.com/guides/concept-testing/；https://contentsquare.com/guides/business-intelligence/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E121" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F121" s="3" t="inlineStr">
         <is>
-          <t>S1-R121-E1 规则：R3-S1-R121-E1-F1 部分验证（候选）（第 2 轮已知 3 个列表链接被匹配但跳到非文章页（/blog/、/guides/ux-design/），是否接受由用户决定）；第 2 轮：候选：R2-CS-BLOG-DETAIL（机械门 passed，留出 6 正 8 反全部正确）——待你确认范围后可升正式；链接 可打开（200，标题「Contentsquare Blog - Digital Experience Insights」）
+          <t>S1-R121-E1 R3-S1-R121-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN5；覆盖检查：列表 277 个、sitemap 同结构 283 个全部匹配
+S1-R121-E1 规则：R3-S1-R121-E1-F1 已验证；第 2 轮：候选：R2-CS-BLOG-DETAIL（机械门 passed，留出 6 正 8 反全部正确）——待你确认范围后可升正式；链接 可打开（200，标题「Contentsquare Blog - Digital Experience Insights」）
 S1-R121-E2 R3-S1-R121-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP3/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
 S1-R121-E2 规则：R3-S1-R121-E2-F1 已验证；链接 可打开（200，标题「Contentsquare eBooks and Reports - Stay Ahead of t」）
 S1-R121-E3 R3-S1-R121-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 50 个、sitemap 同结构 129 个全部匹配
@@ -5895,7 +5910,7 @@
       </c>
       <c r="H121" s="3" t="inlineStr">
         <is>
-          <t>S1-R121-E1: 部分：静态请求 32 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 277；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=9
+          <t>S1-R121-E1: 完整（列表+sitemap 合并枚举）：静态请求 32 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 1 个、成员 277；前缀外同站链接 2、文件 0；sitemap 中同结构但不在列表的 URL：F1=9
   第 2 轮人工复核：部分：静态分页 /blog/page/N/ 共 32 页全部取得（页码连续、无重复页、末页 5 条），唯一详情 277 个；sitemap_index.xml 截断（138 条，止于 f 开头）不能作全集对账，其中 6 篇不在列表；筛选分支未处理；277 篇详情已逐一落地（274 正常、3 跳转到非文章页）；续跑见 output/round3/queue.json
 S1-R121-E2: 完整（枚举结束，无独立全集对账）：静态请求 4 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 140；前缀 /ebooks-reports/ 下家族 1 个、成员 3；前缀外同站链接 27、文件 0；sitemap 中同结构但不在列表的 URL：F1=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -5986,7 +6001,8 @@
         <is>
           <t>^https://blog\.hubspot\.com/marketing/[a-z0-9_-]+$
 ^https://blog\.hubspot\.com/sales/[a-zA-Z0-9%ü-]+$
-^https://blog\.hubspot\.com/service/[a-z0-9-]+$</t>
+^https://blog\.hubspot\.com/service/[a-z0-9-]+$
+^https://blog\.hubspot\.com/website/[a-z0-9_-]+$</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -5998,7 +6014,7 @@
 S1-R123-E3: https://blog.hubspot.com/service
   其余 7 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E3.txt
 S1-R123-E4: https://blog.hubspot.com/website
-  其余 1347 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E4.txt
+  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E4.txt
 S1-R123-E5: https://www.hubspot.com/resources
   其余 56 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R123-E5.txt</t>
         </is>
@@ -6007,12 +6023,13 @@
         <is>
           <t>S1-R123-E1 R3-S1-R123-E1-F1: https://blog.hubspot.com/marketing/ai-search-presence；https://blog.hubspot.com/marketing/gain-instagram-followers（已落地核验 200，公开访问，2026-10-26）
 S1-R123-E2 R3-S1-R123-E2-F1: https://blog.hubspot.com/sales/ai-franchise；https://blog.hubspot.com/sales/avoid-burnout-q4（已落地核验 200，公开访问，2026-10-26）
-S1-R123-E3 R3-S1-R123-E3-F1: https://blog.hubspot.com/service/apology-letter-to-customers；https://blog.hubspot.com/service/customer-success-metrics（已落地核验 200，公开访问，2026-10-26）</t>
+S1-R123-E3 R3-S1-R123-E3-F1: https://blog.hubspot.com/service/apology-letter-to-customers；https://blog.hubspot.com/service/customer-success-metrics（已落地核验 200，公开访问，2026-10-26）
+S1-R123-E4 R3-S1-R123-E4-F1: https://blog.hubspot.com/website/best-woocommerce-product-slider-plugins；https://blog.hubspot.com/website/avoid-ai-credit-overages（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E123" s="3" t="inlineStr">
         <is>
-          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 链接保留；E5 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留；E4 正则+链接保留；E5 链接保留</t>
         </is>
       </c>
       <c r="F123" s="3" t="inlineStr">
@@ -6023,7 +6040,8 @@
 S1-R123-E2 规则：R3-S1-R123-E2-F1 已验证；链接 可打开（200，标题「The HubSpot Sales Blog」）
 S1-R123-E3 R3-S1-R123-E3-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(later_pagination_pages) TP6/FP0/FN0/TN4；覆盖检查：列表 774 个、sitemap 同结构 774 个全部匹配
 S1-R123-E3 规则：R3-S1-R123-E3-F1 已验证；链接 可打开（200，标题「The HubSpot Customer Service Blog」）
-S1-R123-E4 规则：R3-S1-R123-E4-F1 部分验证（候选）（归纳样本跳到家族外页面 2：https://blog.hubspot.com/website/html-elements → https://blog.hubspot.com/website；https://blog.hubspot.com/website/html-span → https://blog.hubspot.com/website）；链接 可打开（200，标题「The HubSpot Website Blog」）
+S1-R123-E4 R3-S1-R123-E4-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(later_pagination_pages) TP6/FP0/FN0/TN4；覆盖检查：列表 1341 个、sitemap 同结构 1338 个全部匹配
+S1-R123-E4 规则：R3-S1-R123-E4-F1 已验证；链接 可打开（200，标题「The HubSpot Website Blog」）
 S1-R123-E5 规则：无规则；链接 可打开（200，标题「Free Resources from HubSpot | Templates, Ebooks, &amp;」）</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Close round-3 gaps: adopt 6 small-sample entries, fix slash and anchor handling
- User decision (2026-10-27): adopt rules without an independent holdout for
  MSI, wearehuman8, Greenbook GRIT, NRF x2, Landor; only that check is waived
  (NRF x2 and Landor now pass full verification anyway)
- Trailing-slash forms count as one family only when the rule's own samples
  show they redirect to each other (GWI /reports/{slug}/ guide pages are a
  different page type)
- Plain in-page anchors in sitemap URLs are not separate pages (IAB)
- DPAA omnichannel study: single landing page, no sub-pages
- Pew sitemap: unescape &amp; in child sitemap URLs (traversal re-running)
- List of the 45 blocked entries: output/round3/blocked-45.xlsx|csv

220 of 268 entries complete; 154 rules in the pattern column (3 adopted).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HW9kjaADHDgTyps9HbQ9Ce
</commit_message>
<xml_diff>
--- a/url-pattern-verification/output/round3/result-table.xlsx
+++ b/url-pattern-verification/output/round3/result-table.xlsx
@@ -1233,7 +1233,7 @@
           <t>S1-R19-E1 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「IP Resources」）
 S1-R19-E2 规则：无规则；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「WIPO Publications」）
 S1-R19-E3 规则：R3-S1-R19-E3-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Intellectual Property Statistics」）
-S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E4-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
+S1-R19-E4 规则：R3-S1-R19-E4-F1 部分验证（候选）（机械门未通过：归纳正例 2&lt;3）；R3-S1-R19-E4-F2 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「PATENTSCOPE」）
 S1-R19-E6 R3-S1-R19-E6-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(other_entries_pages) TP3/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 0 个全部匹配
 S1-R19-E6 规则：R3-S1-R19-E6-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；R3-S1-R19-E6-F2 已验证；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Brand Database」）
 S1-R19-E8 规则：R3-S1-R19-E8-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则（门户页，下级为异构子页面，归属待定）；链接 可打开（200，标题「Global Design Database」）
@@ -1854,25 +1854,34 @@
 https://msi.org/research/</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr"/>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>^https://msi\.org/research/[a-z0-9-]+/$</t>
+        </is>
+      </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
           <t>S1-R31-E1: https://msi.org/library/
   其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R31-E1.txt
 S1-R31-E2: https://msi.org/research/
-  其余 18 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R31-E2.txt</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="inlineStr"/>
+  其余 12 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R31-E2.txt</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>S1-R31-E2 R3-S1-R31-E2-F1: https://msi.org/research/clayton-dissertation-proposal-competition/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
           <t>S1-R31-E1 规则：无规则；链接 可打开（200，标题「Library - MSI」）
-S1-R31-E2 规则：R3-S1-R31-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Research - MSI」）</t>
+S1-R31-E2 R3-S1-R31-E2-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）：node-re2 1.24.1 + google-re2 1.1.20251105 上归纳/回归测试全部通过，覆盖检查无漏配；没有独立留出样本
+S1-R31-E2 规则：R3-S1-R31-E2-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）；链接 可打开（200，标题「Research - MSI」）</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1885,7 +1894,7 @@
         <is>
           <t>S1-R31-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 82；前缀 /library/ 下家族 0 个、成员 0；前缀外同站链接 12、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R31-E2: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 1 个、成员 6；前缀外同站链接 10、文件 2；sitemap 中同结构但不在列表的 URL：F1=5
+S1-R31-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /research/ 下家族 1 个、成员 6；前缀外同站链接 10、文件 2；sitemap 中同结构但不在列表的 URL：F1=5
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -2241,7 +2250,8 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.gwi\.com/blog/[a-z0-9-]+$
+          <t>^https://www\.gwi\.com/reports/[a-z0-9-]+$
+^https://www\.gwi\.com/blog/[a-z0-9-]+$
 ^https://www\.gwi\.com/blog/tag/[a-z-]+$
 ^https://www\.gwi\.com/case\-studies/[a-z0-9-]+$</t>
         </is>
@@ -2249,7 +2259,7 @@
       <c r="C39" s="3" t="inlineStr">
         <is>
           <t>S1-R39-E1: https://www.gwi.com/reports
-  其余 108 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E1.txt
+  其余 10 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E1.txt
 S1-R39-E2: https://www.gwi.com/blog
   其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R39-E2.txt
 S1-R39-E3: https://www.gwi.com/case-studies
@@ -2258,19 +2268,21 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>S1-R39-E2 R3-S1-R39-E2-F1: https://www.gwi.com/blog/brand-purpose；https://www.gwi.com/blog/2025-predictions-vs-reality（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R39-E1 R3-S1-R39-E1-F1: https://www.gwi.com/reports/b2b-in-2021-b；https://www.gwi.com/reports/beauty-buyers（已落地核验 200，公开访问，2026-10-26）
+S1-R39-E2 R3-S1-R39-E2-F1: https://www.gwi.com/blog/brand-purpose；https://www.gwi.com/blog/2025-predictions-vs-reality（已落地核验 200，公开访问，2026-10-26）
 S1-R39-E2 R3-S1-R39-E2-F2: https://www.gwi.com/blog/tag/consumer-behavior；https://www.gwi.com/blog/tag/data-journalism（已落地核验 200，公开访问，2026-10-26）
 S1-R39-E3 R3-S1-R39-E3-F1: https://www.gwi.com/case-studies/conde-nast；https://www.gwi.com/case-studies/barefoot-proximity（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>S1-R39-E1 规则：R3-S1-R39-E1-F1 部分验证（候选）（机械门未通过：标注测试有失败（留出 FN0/FP0））；链接 可打开（200，标题「Reports - Resources, Marketing Infographics &amp; Guid」）
+          <t>S1-R39-E1 R3-S1-R39-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 98 个、sitemap 同结构 92 个全部匹配
+S1-R39-E1 规则：R3-S1-R39-E1-F1 已验证；链接 可打开（200，标题「Reports - Resources, Marketing Infographics &amp; Guid」）
 S1-R39-E2 R3-S1-R39-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 21 个、sitemap 同结构 458 个全部匹配
 S1-R39-E2 R3-S1-R39-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP1/FP0/FN0/TN7；覆盖检查：列表 7 个、sitemap 同结构 0 个全部匹配
 S1-R39-E2 规则：R3-S1-R39-E2-F1 已验证；R3-S1-R39-E2-F2 已验证；链接 可打开（200，标题「Digital &amp; Social Trends, Charts, Consumer Data &amp; S」）
@@ -2287,7 +2299,7 @@
       </c>
       <c r="H39" s="3" t="inlineStr">
         <is>
-          <t>S1-R39-E1: 部分：静态请求 12 页（入口+分页），未完成分页 0；前缀 /reports/ 下家族 1 个、成员 98；前缀外同站链接 8、文件 0；sitemap 中同结构但不在列表的 URL：F1=21
+          <t>S1-R39-E1: 完整（列表+sitemap 合并枚举）：静态请求 12 页（入口+分页），未完成分页 0；前缀 /reports/ 下家族 1 个、成员 98；前缀外同站链接 8、文件 0；sitemap 中同结构但不在列表的 URL：F1=20
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R39-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 28；前缀外同站链接 6、文件 0；sitemap 中同结构但不在列表的 URL：F1=437、F2=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
@@ -2307,22 +2319,31 @@
           <t>https://www.wearehuman8.com/inspiration/</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.wearehuman8\.com/inspiration/[a-z-]+/$</t>
+        </is>
+      </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>S1-R40-E1: https://www.wearehuman8.com/inspiration/
-  其余 295 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R40-E1.txt</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr"/>
+  其余 291 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R40-E1.txt</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>S1-R40-E1 R3-S1-R40-E1-F1: https://www.wearehuman8.com/inspiration/reports-ebooks/；https://www.wearehuman8.com/inspiration/blog/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>S1-R40-E1 规则：R3-S1-R40-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Inspiration - Human8」）</t>
+          <t>S1-R40-E1 R3-S1-R40-E1-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）：node-re2 1.24.1 + google-re2 1.1.20251105 上归纳/回归测试全部通过，覆盖检查无漏配；没有独立留出样本
+S1-R40-E1 规则：R3-S1-R40-E1-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）；链接 可打开（200，标题「Inspiration - Human8」）</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -2332,7 +2353,7 @@
       </c>
       <c r="H40" s="3" t="inlineStr">
         <is>
-          <t>S1-R40-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /inspiration/ 下家族 1 个、成员 4；前缀外同站链接 291、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
+          <t>S1-R40-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /inspiration/ 下家族 1 个、成员 4；前缀外同站链接 291、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -3547,24 +3568,33 @@
 https://www.iab.com/get-involved/</t>
         </is>
       </c>
-      <c r="B68" s="4" t="inlineStr"/>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>^https://www\.iab\.com/events/[a-z0-9_-]+/$</t>
+        </is>
+      </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
           <t>S1-R68-E1: https://www.iab.com/events/
-  其余 84 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R68-E1.txt
+  其余 65 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R68-E1.txt
 S1-R68-E2: https://www.iab.com/get-involved/
   其余 10 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R68-E2.txt</t>
         </is>
       </c>
-      <c r="D68" s="3" t="inlineStr"/>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>S1-R68-E1 R3-S1-R68-E1-F1: https://www.iab.com/events/2019-iab-global-summit/；https://www.iab.com/events/beyond-iab-creatorfronts-whats-next-for-creator-marketing/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 正则+链接保留；E2 链接保留</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>S1-R68-E1 规则：R3-S1-R68-E1-F1 部分验证（候选）（sitemap 同结构 URL 漏配 4）；链接 可打开（200，标题「Events」）
+          <t>S1-R68-E1 R3-S1-R68-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN4；覆盖检查：列表 19 个、sitemap 同结构 961 个全部匹配
+S1-R68-E1 规则：R3-S1-R68-E1-F1 已验证；链接 可打开（200，标题「Events」）
 S1-R68-E2 规则：无规则；链接 可打开（200，标题「Interactive Advertising Bureau | Become A Member」）</t>
         </is>
       </c>
@@ -3576,7 +3606,7 @@
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
-          <t>S1-R68-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 535；前缀 /events/ 下家族 1 个、成员 19；前缀外同站链接 65、文件 0；sitemap 中同结构但不在列表的 URL：F1=946
+          <t>S1-R68-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 535；前缀 /events/ 下家族 1 个、成员 19；前缀外同站链接 65、文件 0；sitemap 中同结构但不在列表的 URL：F1=943
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R68-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 173；前缀 /get-involved/ 下家族 0 个、成员 0；前缀外同站链接 10、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -4381,7 +4411,8 @@
       </c>
       <c r="H88" s="3" t="inlineStr">
         <is>
-          <t>S1-R88-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 44；前缀 /omnichannel-study/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；页面上没有可枚举的标准链接（a[href]），内容可能由脚本组件渲染
+          <t>S1-R88-E1: 完整：单页活动落地页：页面链接只有页内锚点（#About、#Resources）、站外/其他研究页和 1 个文件，入口前缀 /omnichannel-study/ 下没有子页面（静态与浏览器渲染一致）
+  部分：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 44；前缀 /omnichannel-study/ 下家族 0 个、成员 0；前缀外同站链接 0、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）；页面上没有可枚举的标准链接（a[href]），内容可能由脚本组件渲染
   第 2 轮人工复核：部分：入口静态首轮 1 页（2189 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -4403,7 +4434,8 @@
       <c r="B89" s="4" t="inlineStr">
         <is>
           <t>^https://www\.greenbook\.org/insights/[a-z0-9-]+/[a-z0-9-]+$
-^https://www\.greenbook\.org/insights/[a-z0-9_-]+$</t>
+^https://www\.greenbook\.org/insights/[a-z0-9_-]+$
+^https://www\.greenbook\.org/grit/[a-z0-9-]+$</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -4413,18 +4445,19 @@
 S1-R89-E2: https://www.greenbook.org/insights
   其余 39 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R89-E2.txt
 S1-R89-E3: https://www.greenbook.org/grit
-  其余 13 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R89-E3.txt</t>
+  其余 10 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R89-E3.txt</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
           <t>S1-R89-E2 R3-S1-R89-E2-F1: https://www.greenbook.org/insights/artificial-intelligence-and-machine-learning/how-to-get-real-insights-from-synthetic-personas；https://www.greenbook.org/insights/artificial-intelligence-and-machine-learning/beyond-synthetic-consumers-building-a-human-ai-model-for-better-brand-decisions（已落地核验 200，公开访问，2026-10-26）
-S1-R89-E2 R3-S1-R89-E2-F2: https://www.greenbook.org/insights/empowered-to-lead-with-empathy-how-experian-health-used-alida-to-discover-and-act-on-voc-and-voe；https://www.greenbook.org/insights/data-quality-privacy-and-ethics（已落地核验 200，公开访问，2026-10-26）</t>
+S1-R89-E2 R3-S1-R89-E2-F2: https://www.greenbook.org/insights/empowered-to-lead-with-empathy-how-experian-health-used-alida-to-discover-and-act-on-voc-and-voe；https://www.greenbook.org/insights/data-quality-privacy-and-ethics（已落地核验 200，公开访问，2026-10-26）
+S1-R89-E3 R3-S1-R89-E3-F1: https://www.greenbook.org/grit/grit-business-and-innovation-edition（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 正则+链接保留；E3 链接保留</t>
+          <t>E1 链接保留；E2 正则+链接保留；E3 正则+链接保留</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -4433,7 +4466,8 @@
 S1-R89-E2 R3-S1-R89-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 66 个、sitemap 同结构 5213 个全部匹配
 S1-R89-E2 R3-S1-R89-E2-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 36 个、sitemap 同结构 847 个全部匹配
 S1-R89-E2 规则：R3-S1-R89-E2-F1 已验证；R3-S1-R89-E2-F2 已验证；第 2 轮：无规则；链接 可打开（200，标题「Insights — Greenbook」）
-S1-R89-E3 规则：R3-S1-R89-E3-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；第 2 轮：无规则；链接 可打开（200，标题「GRIT — Greenbook」）</t>
+S1-R89-E3 R3-S1-R89-E3-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）：node-re2 1.24.1 + google-re2 1.1.20251105 上归纳/回归测试全部通过，覆盖检查无漏配；没有独立留出样本
+S1-R89-E3 规则：R3-S1-R89-E3-F1 已采用（用户 2026-10-27 同意：小样本，未经独立留出验证）；第 2 轮：无规则；链接 可打开（200，标题「GRIT — Greenbook」）</t>
         </is>
       </c>
       <c r="G89" s="3" t="inlineStr">
@@ -4449,7 +4483,7 @@
   第 2 轮人工复核：部分：入口静态首轮 1 页（4420 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json
 S1-R89-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /insights/ 下家族 2 个、成员 102；前缀外同站链接 39、文件 0；sitemap 中同结构但不在列表的 URL：F1=5147、F2=814
   第 2 轮人工复核：部分：入口静态首轮 1 页（37390 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json
-S1-R89-E3: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /grit/ 下家族 1 个、成员 3；前缀外同站链接 10、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
+S1-R89-E3: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /grit/ 下家族 1 个、成员 3；前缀外同站链接 10、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
   第 2 轮人工复核：部分：入口静态首轮 1 页（16977 字正文，链接已入 edges）；分页/详情/动态未处理；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -5096,25 +5130,37 @@
 https://nrf.com/about-us</t>
         </is>
       </c>
-      <c r="B105" s="4" t="inlineStr"/>
+      <c r="B105" s="4" t="inlineStr">
+        <is>
+          <t>^https://nrf\.com/membership/[a-z-]+$
+^https://nrf\.com/about\-us/[a-z0-9-]+$</t>
+        </is>
+      </c>
       <c r="C105" s="3" t="inlineStr">
         <is>
           <t>S1-R105-E1: https://nrf.com/membership
-  其余 3 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R105-E1.txt
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R105-E1.txt
 S1-R105-E2: https://nrf.com/about-us
-  其余 6 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R105-E2.txt</t>
-        </is>
-      </c>
-      <c r="D105" s="3" t="inlineStr"/>
+  其余 2 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R105-E2.txt</t>
+        </is>
+      </c>
+      <c r="D105" s="3" t="inlineStr">
+        <is>
+          <t>S1-R105-E1 R3-S1-R105-E1-F1: https://nrf.com/membership/current-university-members；https://nrf.com/membership/nrf-industry-partner-membership（已落地核验 200，公开访问，2026-10-26）
+S1-R105-E2 R3-S1-R105-E2-F1: https://nrf.com/about-us/2024；https://nrf.com/about-us/2025（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E105" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留；E2 链接保留</t>
+          <t>E1 正则+链接保留；E2 正则+链接保留</t>
         </is>
       </c>
       <c r="F105" s="3" t="inlineStr">
         <is>
-          <t>S1-R105-E1 规则：R3-S1-R105-E1-F1 链接保留（仅 3 个同结构目标，按技能不强凑正则）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「NRF Membership | NRF」）
-S1-R105-E2 规则：R3-S1-R105-E2-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「About the National Retail Federation | NRF」）</t>
+          <t>S1-R105-E1 R3-S1-R105-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP1/FP0/FN0/TN5；覆盖检查：列表 3 个、sitemap 同结构 4 个全部匹配
+S1-R105-E1 规则：R3-S1-R105-E1-F1 已验证；链接 可打开（200，标题「NRF Membership | NRF」）
+S1-R105-E2 R3-S1-R105-E2-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP5/FP0/FN0/TN6；覆盖检查：列表 4 个、sitemap 同结构 8 个全部匹配
+S1-R105-E2 规则：R3-S1-R105-E2-F1 已验证；链接 可打开（200，标题「About the National Retail Federation | NRF」）</t>
         </is>
       </c>
       <c r="G105" s="3" t="inlineStr">
@@ -5125,9 +5171,9 @@
       </c>
       <c r="H105" s="3" t="inlineStr">
         <is>
-          <t>S1-R105-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /membership/ 下家族 1 个、成员 3；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=3
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R105-E2: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /about-us/ 下家族 1 个、成员 4；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=6
+          <t>S1-R105-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /membership/ 下家族 1 个、成员 3；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=1
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R105-E2: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /about-us/ 下家族 1 个、成员 4；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=5
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -5803,7 +5849,7 @@
       </c>
       <c r="B120" s="4" t="inlineStr">
         <is>
-          <t>^https://buffer\.com/resources/[a-z0-9-]+/?$
+          <t>^https://buffer\.com/resources/[a-z0-9-]+/$
 ^https://buffer\.com/resources/author/[a-z0-9-]+/$</t>
         </is>
       </c>
@@ -5817,7 +5863,7 @@
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>S1-R120-E1 R3-S1-R120-E1-F1: https://buffer.com/resources/5-simple-seo-tactics/；https://buffer.com/resources/how-buffer-helped-me-triple-my-linkedin-impressions-and-grow-my-newsletter/（已落地核验 200，公开访问，2026-10-26）
+          <t>S1-R120-E1 R3-S1-R120-E1-F1: https://buffer.com/resources/culturelab-podcast/；https://buffer.com/resources/how-buffer-helped-me-triple-my-linkedin-impressions-and-grow-my-newsletter/（已落地核验 200，公开访问，2026-10-26）
 S1-R120-E1 R3-S1-R120-E1-F2: https://buffer.com/resources/author/amanda-holliday/；https://buffer.com/resources/author/eric-lam/（已落地核验 200，公开访问，2026-10-26）</t>
         </is>
       </c>
@@ -5828,7 +5874,7 @@
       </c>
       <c r="F120" s="3" t="inlineStr">
         <is>
-          <t>S1-R120-E1 R3-S1-R120-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 155 个、sitemap 同结构 2490 个全部匹配
+          <t>S1-R120-E1 R3-S1-R120-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN7；覆盖检查：列表 155 个、sitemap 同结构 2488 个全部匹配
 S1-R120-E1 R3-S1-R120-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 23 个、sitemap 同结构 330 个全部匹配
 S1-R120-E1 规则：R3-S1-R120-E1-F1 已验证；R3-S1-R120-E1-F2 已验证；链接 可打开（200，标题「Buffer Blog - Thoughts on Social Media &amp; Online Ma」）
 S1-R120-E2 规则：无规则；链接 可打开（200，标题「Buffer’s Social Media and Marketing Library」）</t>
@@ -5842,7 +5888,7 @@
       </c>
       <c r="H120" s="3" t="inlineStr">
         <is>
-          <t>S1-R120-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 2 个、成员 178；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=2336、F2=307
+          <t>S1-R120-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /resources/ 下家族 2 个、成员 178；前缀外同站链接 1、文件 0；sitemap 中同结构但不在列表的 URL：F1=2334、F2=307
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R120-E2: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 238；前缀 /library/ 下家族 0 个、成员 0；前缀外同站链接 33、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
@@ -6203,22 +6249,31 @@
           <t>https://landor.com/en/our-work/</t>
         </is>
       </c>
-      <c r="B126" s="4" t="inlineStr"/>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>^https://landor\.com/en/our\-work/[a-z0-9-]+/$</t>
+        </is>
+      </c>
       <c r="C126" s="3" t="inlineStr">
         <is>
           <t>S1-R126-E1: https://landor.com/en/our-work/
-  其余 38 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R126-E1.txt</t>
-        </is>
-      </c>
-      <c r="D126" s="3" t="inlineStr"/>
+  其余 0 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R126-E1.txt</t>
+        </is>
+      </c>
+      <c r="D126" s="3" t="inlineStr">
+        <is>
+          <t>S1-R126-E1 R3-S1-R126-E1-F1: https://landor.com/en/our-work/bancomat/；https://landor.com/en/our-work/ao/（已落地核验 200，公开访问，2026-10-26）</t>
+        </is>
+      </c>
       <c r="E126" s="3" t="inlineStr">
         <is>
-          <t>E1 链接保留</t>
+          <t>E1 正则+链接保留</t>
         </is>
       </c>
       <c r="F126" s="3" t="inlineStr">
         <is>
-          <t>S1-R126-E1 规则：R3-S1-R126-E1-F1 部分验证（候选）（机械门未通过：无独立留出正例（sitemap、后续分页、其他页面、详情页链接均无同结构样本））；链接 可打开（200，标题「Our work」）</t>
+          <t>S1-R126-E1 R3-S1-R126-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP6/FP0/FN0/TN5；覆盖检查：列表 38 个、sitemap 同结构 0 个全部匹配
+S1-R126-E1 规则：R3-S1-R126-E1-F1 已验证；链接 可打开（200，标题「Our work」）</t>
         </is>
       </c>
       <c r="G126" s="3" t="inlineStr">
@@ -6228,7 +6283,7 @@
       </c>
       <c r="H126" s="3" t="inlineStr">
         <is>
-          <t>S1-R126-E1: 部分：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/our-work/ 下家族 1 个、成员 38；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=38
+          <t>S1-R126-E1: 完整（枚举结束，无独立全集对账）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /en/our-work/ 下家族 1 个、成员 38；前缀外同站链接 0、文件 0；sitemap 中同结构但不在列表的 URL：F1=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>
@@ -6668,14 +6723,14 @@
       </c>
       <c r="B135" s="4" t="inlineStr">
         <is>
-          <t>^https://www\.sistrix\.com/blog/[a-z0-9%_-]+/?$
+          <t>^https://www\.sistrix\.com/blog/[a-z0-9%_-]+/$
 ^https://www\.sistrix\.com/blog/archive/\?selected=[0-9]*$</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
         <is>
           <t>S1-R135-E1: https://www.sistrix.com/blog/
-  其余 24 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R135-E1.txt</t>
+  其余 25 个未被正式规则覆盖的已知目标见 output/round3/retained/S1-R135-E1.txt</t>
         </is>
       </c>
       <c r="D135" s="3" t="inlineStr">
@@ -6691,7 +6746,7 @@
       </c>
       <c r="F135" s="3" t="inlineStr">
         <is>
-          <t>S1-R135-E1 R3-S1-R135-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 25 个、sitemap 同结构 840 个全部匹配
+          <t>S1-R135-E1 R3-S1-R135-E1-F1 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(sitemap) TP6/FP0/FN0/TN6；覆盖检查：列表 25 个、sitemap 同结构 836 个全部匹配
 S1-R135-E1 R3-S1-R135-E1-F2 已验证：node-re2 1.24.1 + google-re2 1.1.20251105 逐对一致；留出(listing_split) TP5/FP0/FN0/TN7；覆盖检查：列表 20 个、sitemap 同结构 0 个全部匹配
 S1-R135-E1 规则：R3-S1-R135-E1-F1 已验证；R3-S1-R135-E1-F2 已验证；链接 可打开（200，标题「SISTRIX SEO Blog, studies and expert content - SIS」）</t>
         </is>
@@ -6703,7 +6758,7 @@
       </c>
       <c r="H135" s="3" t="inlineStr">
         <is>
-          <t>S1-R135-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 45；前缀外同站链接 24、文件 0；sitemap 中同结构但不在列表的 URL：F1=815、F2=0
+          <t>S1-R135-E1: 完整（列表+sitemap 合并枚举）：静态请求 1 页（入口+分页），未完成分页 0；前缀 /blog/ 下家族 2 个、成员 45；前缀外同站链接 24、文件 0；sitemap 中同结构但不在列表的 URL：F1=811、F2=0
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Finish Pew sitemap traversal; 222 of 268 entries complete
Pew sitemap fully traversed (405 rate-limited files retried slowly, 404 ok,
1 real 404); no URLs under the two /topic/ entries, so both are complete.
Remaining: 45 blocked entries (list in output/round3/blocked-45.xlsx) and
Circana Insights (Wix page without standard links).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HW9kjaADHDgTyps9HbQ9Ce
</commit_message>
<xml_diff>
--- a/url-pattern-verification/output/round3/result-table.xlsx
+++ b/url-pattern-verification/output/round3/result-table.xlsx
@@ -3068,9 +3068,9 @@
         <is>
           <t>S1-R52-E1: 完整（枚举结束，无独立全集对账）：静态请求 6 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 129；前缀 /topic/economy-work/ 下家族 1 个、成员 3；前缀外同站链接 30、文件 0；sitemap 中同结构但不在列表的 URL：F1=0；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R52-E2: 部分：静态请求 4 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 145；前缀 /topic/internet-technology/ 下家族 1 个、成员 4；前缀外同站链接 21、文件 0；sitemap 中同结构但不在列表的 URL：F1=27；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
-  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
-S1-R52-E3: 部分：静态请求 7 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 147；前缀 /topic/news-habits-media/ 下家族 1 个、成员 5；前缀外同站链接 41、文件 0；sitemap 中同结构但不在列表的 URL：F1=11；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+S1-R52-E2: 完整（列表+sitemap 合并枚举）：静态请求 4 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 145；前缀 /topic/internet-technology/ 下家族 1 个、成员 4；前缀外同站链接 21、文件 0；sitemap 中同结构但不在列表的 URL：F1=27；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
+  第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
+S1-R52-E3: 完整（列表+sitemap 合并枚举）：静态请求 7 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 147；前缀 /topic/news-habits-media/ 下家族 1 个、成员 5；前缀外同站链接 41、文件 0；sitemap 中同结构但不在列表的 URL：F1=11；内容区无前缀内链接，栏目条目取自页面 nav/header 中的前缀内链接
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json
 S1-R52-E4: 完整（枚举结束，无独立全集对账）：静态请求 15 页（入口+分页），未完成分页 0；浏览器渲染 2 轮、点击加载更多 0 次、渲染后链接 120；前缀 /topic/economy-work/business-workplace/ 下家族 0 个、成员 0；前缀外同站链接 85、文件 0；未发现可归纳的下级家族（下级链接不足 3 个同结构或均在前缀外）
   第 2 轮人工复核：未验证：本轮只处理优先级 1；仅做 host 级连通性测试；续跑见 output/round3/queue.json</t>

</xml_diff>